<commit_message>
Verify bank-funding exposure against Q2 FY24 filings; move filings to filings/; H1 RBI checks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QUxicXQrqdyqQxohnFLPv8
</commit_message>
<xml_diff>
--- a/Dissertation_Data.xlsx
+++ b/Dissertation_Data.xlsx
@@ -622,7 +622,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>1 if Bank_Exposure above median (55.0%)</t>
+          <t>1 if Bank_Exposure above median (54.6%)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
-        <v>44.5</v>
+        <v>49.6</v>
       </c>
       <c r="Q2" t="n">
         <v>0</v>
@@ -909,7 +909,7 @@
         <v>18.2766</v>
       </c>
       <c r="P3" t="n">
-        <v>44.5</v>
+        <v>49.6</v>
       </c>
       <c r="Q3" t="n">
         <v>0</v>
@@ -973,7 +973,7 @@
         <v>22.1659</v>
       </c>
       <c r="P4" t="n">
-        <v>44.5</v>
+        <v>49.6</v>
       </c>
       <c r="Q4" t="n">
         <v>0</v>
@@ -1037,7 +1037,7 @@
         <v>20.054</v>
       </c>
       <c r="P5" t="n">
-        <v>44.5</v>
+        <v>49.6</v>
       </c>
       <c r="Q5" t="n">
         <v>0</v>
@@ -1046,7 +1046,7 @@
         <v>1</v>
       </c>
       <c r="S5" t="n">
-        <v>44.5</v>
+        <v>49.6</v>
       </c>
       <c r="T5" t="n">
         <v>6.5</v>
@@ -1101,7 +1101,7 @@
         <v>16.509</v>
       </c>
       <c r="P6" t="n">
-        <v>44.5</v>
+        <v>49.6</v>
       </c>
       <c r="Q6" t="n">
         <v>0</v>
@@ -1110,7 +1110,7 @@
         <v>1</v>
       </c>
       <c r="S6" t="n">
-        <v>44.5</v>
+        <v>49.6</v>
       </c>
       <c r="T6" t="n">
         <v>6.4632</v>
@@ -1165,7 +1165,7 @@
         <v>13.8418</v>
       </c>
       <c r="P7" t="n">
-        <v>44.5</v>
+        <v>49.6</v>
       </c>
       <c r="Q7" t="n">
         <v>0</v>
@@ -1174,7 +1174,7 @@
         <v>1</v>
       </c>
       <c r="S7" t="n">
-        <v>44.5</v>
+        <v>49.6</v>
       </c>
       <c r="T7" t="n">
         <v>5.5153</v>
@@ -1227,10 +1227,10 @@
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="n">
-        <v>71</v>
+        <v>32.3</v>
       </c>
       <c r="Q8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -1291,10 +1291,10 @@
         <v>45.1777</v>
       </c>
       <c r="P9" t="n">
-        <v>71</v>
+        <v>32.3</v>
       </c>
       <c r="Q9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
@@ -1355,10 +1355,10 @@
         <v>45.4783</v>
       </c>
       <c r="P10" t="n">
-        <v>71</v>
+        <v>32.3</v>
       </c>
       <c r="Q10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
@@ -1419,16 +1419,16 @@
         <v>30.6167</v>
       </c>
       <c r="P11" t="n">
-        <v>71</v>
+        <v>32.3</v>
       </c>
       <c r="Q11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R11" t="n">
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>71</v>
+        <v>32.3</v>
       </c>
       <c r="T11" t="n">
         <v>6.5</v>
@@ -1483,16 +1483,16 @@
         <v>0.416</v>
       </c>
       <c r="P12" t="n">
-        <v>71</v>
+        <v>32.3</v>
       </c>
       <c r="Q12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R12" t="n">
         <v>1</v>
       </c>
       <c r="S12" t="n">
-        <v>71</v>
+        <v>32.3</v>
       </c>
       <c r="T12" t="n">
         <v>6.4632</v>
@@ -1547,16 +1547,16 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>71</v>
+        <v>32.3</v>
       </c>
       <c r="Q13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R13" t="n">
         <v>1</v>
       </c>
       <c r="S13" t="n">
-        <v>71</v>
+        <v>32.3</v>
       </c>
       <c r="T13" t="n">
         <v>5.5153</v>
@@ -1991,10 +1991,10 @@
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="Q20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R20" t="n">
         <v>0</v>
@@ -2055,10 +2055,10 @@
         <v>18.9272</v>
       </c>
       <c r="P21" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="Q21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R21" t="n">
         <v>0</v>
@@ -2119,10 +2119,10 @@
         <v>16.691</v>
       </c>
       <c r="P22" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="Q22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R22" t="n">
         <v>0</v>
@@ -2183,16 +2183,16 @@
         <v>10.3334</v>
       </c>
       <c r="P23" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="Q23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R23" t="n">
         <v>1</v>
       </c>
       <c r="S23" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="T23" t="n">
         <v>6.5</v>
@@ -2247,16 +2247,16 @@
         <v>8.796099999999999</v>
       </c>
       <c r="P24" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="Q24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R24" t="n">
         <v>1</v>
       </c>
       <c r="S24" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="T24" t="n">
         <v>6.4632</v>
@@ -2311,16 +2311,16 @@
         <v>9.9353</v>
       </c>
       <c r="P25" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="Q25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R25" t="n">
         <v>1</v>
       </c>
       <c r="S25" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="T25" t="n">
         <v>5.5153</v>
@@ -2373,10 +2373,10 @@
       </c>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="n">
-        <v>53.5</v>
+        <v>60</v>
       </c>
       <c r="Q26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R26" t="n">
         <v>0</v>
@@ -2437,10 +2437,10 @@
         <v>49.7395</v>
       </c>
       <c r="P27" t="n">
-        <v>53.5</v>
+        <v>60</v>
       </c>
       <c r="Q27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R27" t="n">
         <v>0</v>
@@ -2501,10 +2501,10 @@
         <v>30.7773</v>
       </c>
       <c r="P28" t="n">
-        <v>53.5</v>
+        <v>60</v>
       </c>
       <c r="Q28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R28" t="n">
         <v>0</v>
@@ -2565,16 +2565,16 @@
         <v>30.9663</v>
       </c>
       <c r="P29" t="n">
-        <v>53.5</v>
+        <v>60</v>
       </c>
       <c r="Q29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R29" t="n">
         <v>1</v>
       </c>
       <c r="S29" t="n">
-        <v>53.5</v>
+        <v>60</v>
       </c>
       <c r="T29" t="n">
         <v>6.5</v>
@@ -2629,16 +2629,16 @@
         <v>21.1904</v>
       </c>
       <c r="P30" t="n">
-        <v>53.5</v>
+        <v>60</v>
       </c>
       <c r="Q30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R30" t="n">
         <v>1</v>
       </c>
       <c r="S30" t="n">
-        <v>53.5</v>
+        <v>60</v>
       </c>
       <c r="T30" t="n">
         <v>6.4632</v>
@@ -2693,16 +2693,16 @@
         <v>16.9076</v>
       </c>
       <c r="P31" t="n">
-        <v>53.5</v>
+        <v>60</v>
       </c>
       <c r="Q31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R31" t="n">
         <v>1</v>
       </c>
       <c r="S31" t="n">
-        <v>53.5</v>
+        <v>60</v>
       </c>
       <c r="T31" t="n">
         <v>5.5153</v>
@@ -2755,10 +2755,10 @@
       </c>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="n">
-        <v>58</v>
+        <v>52.9</v>
       </c>
       <c r="Q32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2819,10 +2819,10 @@
         <v>20.0229</v>
       </c>
       <c r="P33" t="n">
-        <v>58</v>
+        <v>52.9</v>
       </c>
       <c r="Q33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2883,10 +2883,10 @@
         <v>23.6655</v>
       </c>
       <c r="P34" t="n">
-        <v>58</v>
+        <v>52.9</v>
       </c>
       <c r="Q34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2947,16 +2947,16 @@
         <v>23.919</v>
       </c>
       <c r="P35" t="n">
-        <v>58</v>
+        <v>52.9</v>
       </c>
       <c r="Q35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R35" t="n">
         <v>1</v>
       </c>
       <c r="S35" t="n">
-        <v>58</v>
+        <v>52.9</v>
       </c>
       <c r="T35" t="n">
         <v>6.5</v>
@@ -3011,16 +3011,16 @@
         <v>-3.0945</v>
       </c>
       <c r="P36" t="n">
-        <v>58</v>
+        <v>52.9</v>
       </c>
       <c r="Q36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R36" t="n">
         <v>1</v>
       </c>
       <c r="S36" t="n">
-        <v>58</v>
+        <v>52.9</v>
       </c>
       <c r="T36" t="n">
         <v>6.4632</v>
@@ -3075,16 +3075,16 @@
         <v>13.3193</v>
       </c>
       <c r="P37" t="n">
-        <v>58</v>
+        <v>52.9</v>
       </c>
       <c r="Q37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R37" t="n">
         <v>1</v>
       </c>
       <c r="S37" t="n">
-        <v>58</v>
+        <v>52.9</v>
       </c>
       <c r="T37" t="n">
         <v>5.5153</v>
@@ -3137,10 +3137,10 @@
       </c>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="n">
-        <v>57.5</v>
+        <v>54</v>
       </c>
       <c r="Q38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -3201,10 +3201,10 @@
         <v>26.1783</v>
       </c>
       <c r="P39" t="n">
-        <v>57.5</v>
+        <v>54</v>
       </c>
       <c r="Q39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3265,10 +3265,10 @@
         <v>29.1059</v>
       </c>
       <c r="P40" t="n">
-        <v>57.5</v>
+        <v>54</v>
       </c>
       <c r="Q40" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3329,16 +3329,16 @@
         <v>29.8096</v>
       </c>
       <c r="P41" t="n">
-        <v>57.5</v>
+        <v>54</v>
       </c>
       <c r="Q41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R41" t="n">
         <v>1</v>
       </c>
       <c r="S41" t="n">
-        <v>57.5</v>
+        <v>54</v>
       </c>
       <c r="T41" t="n">
         <v>6.5</v>
@@ -3393,16 +3393,16 @@
         <v>27.0702</v>
       </c>
       <c r="P42" t="n">
-        <v>57.5</v>
+        <v>54</v>
       </c>
       <c r="Q42" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R42" t="n">
         <v>1</v>
       </c>
       <c r="S42" t="n">
-        <v>57.5</v>
+        <v>54</v>
       </c>
       <c r="T42" t="n">
         <v>6.4632</v>
@@ -3457,16 +3457,16 @@
         <v>22.2314</v>
       </c>
       <c r="P43" t="n">
-        <v>57.5</v>
+        <v>54</v>
       </c>
       <c r="Q43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R43" t="n">
         <v>1</v>
       </c>
       <c r="S43" t="n">
-        <v>57.5</v>
+        <v>54</v>
       </c>
       <c r="T43" t="n">
         <v>5.5153</v>
@@ -3519,7 +3519,7 @@
       </c>
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="n">
-        <v>56</v>
+        <v>55.3</v>
       </c>
       <c r="Q44" t="n">
         <v>1</v>
@@ -3583,7 +3583,7 @@
         <v>13.623</v>
       </c>
       <c r="P45" t="n">
-        <v>56</v>
+        <v>55.3</v>
       </c>
       <c r="Q45" t="n">
         <v>1</v>
@@ -3647,7 +3647,7 @@
         <v>23.2868</v>
       </c>
       <c r="P46" t="n">
-        <v>56</v>
+        <v>55.3</v>
       </c>
       <c r="Q46" t="n">
         <v>1</v>
@@ -3711,7 +3711,7 @@
         <v>20.0139</v>
       </c>
       <c r="P47" t="n">
-        <v>56</v>
+        <v>55.3</v>
       </c>
       <c r="Q47" t="n">
         <v>1</v>
@@ -3720,7 +3720,7 @@
         <v>1</v>
       </c>
       <c r="S47" t="n">
-        <v>56</v>
+        <v>55.3</v>
       </c>
       <c r="T47" t="n">
         <v>6.5</v>
@@ -3775,7 +3775,7 @@
         <v>-0.787</v>
       </c>
       <c r="P48" t="n">
-        <v>56</v>
+        <v>55.3</v>
       </c>
       <c r="Q48" t="n">
         <v>1</v>
@@ -3784,7 +3784,7 @@
         <v>1</v>
       </c>
       <c r="S48" t="n">
-        <v>56</v>
+        <v>55.3</v>
       </c>
       <c r="T48" t="n">
         <v>6.4632</v>
@@ -3839,7 +3839,7 @@
         <v>26.3902</v>
       </c>
       <c r="P49" t="n">
-        <v>56</v>
+        <v>55.3</v>
       </c>
       <c r="Q49" t="n">
         <v>1</v>
@@ -3848,7 +3848,7 @@
         <v>1</v>
       </c>
       <c r="S49" t="n">
-        <v>56</v>
+        <v>55.3</v>
       </c>
       <c r="T49" t="n">
         <v>5.5153</v>
@@ -3901,7 +3901,7 @@
       </c>
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="n">
-        <v>24.5</v>
+        <v>33</v>
       </c>
       <c r="Q50" t="n">
         <v>0</v>
@@ -3965,7 +3965,7 @@
         <v>7.9181</v>
       </c>
       <c r="P51" t="n">
-        <v>24.5</v>
+        <v>33</v>
       </c>
       <c r="Q51" t="n">
         <v>0</v>
@@ -4029,7 +4029,7 @@
         <v>9.101100000000001</v>
       </c>
       <c r="P52" t="n">
-        <v>24.5</v>
+        <v>33</v>
       </c>
       <c r="Q52" t="n">
         <v>0</v>
@@ -4093,7 +4093,7 @@
         <v>4.1843</v>
       </c>
       <c r="P53" t="n">
-        <v>24.5</v>
+        <v>33</v>
       </c>
       <c r="Q53" t="n">
         <v>0</v>
@@ -4102,7 +4102,7 @@
         <v>1</v>
       </c>
       <c r="S53" t="n">
-        <v>24.5</v>
+        <v>33</v>
       </c>
       <c r="T53" t="n">
         <v>6.5</v>
@@ -4157,7 +4157,7 @@
         <v>4.8325</v>
       </c>
       <c r="P54" t="n">
-        <v>24.5</v>
+        <v>33</v>
       </c>
       <c r="Q54" t="n">
         <v>0</v>
@@ -4166,7 +4166,7 @@
         <v>1</v>
       </c>
       <c r="S54" t="n">
-        <v>24.5</v>
+        <v>33</v>
       </c>
       <c r="T54" t="n">
         <v>6.4632</v>
@@ -4221,7 +4221,7 @@
         <v>5.4941</v>
       </c>
       <c r="P55" t="n">
-        <v>24.5</v>
+        <v>33</v>
       </c>
       <c r="Q55" t="n">
         <v>0</v>
@@ -4230,7 +4230,7 @@
         <v>1</v>
       </c>
       <c r="S55" t="n">
-        <v>24.5</v>
+        <v>33</v>
       </c>
       <c r="T55" t="n">
         <v>5.5153</v>
@@ -4283,7 +4283,7 @@
       </c>
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="n">
-        <v>56.5</v>
+        <v>57.2</v>
       </c>
       <c r="Q56" t="n">
         <v>1</v>
@@ -4347,7 +4347,7 @@
         <v>1.0921</v>
       </c>
       <c r="P57" t="n">
-        <v>56.5</v>
+        <v>57.2</v>
       </c>
       <c r="Q57" t="n">
         <v>1</v>
@@ -4411,7 +4411,7 @@
         <v>11.8759</v>
       </c>
       <c r="P58" t="n">
-        <v>56.5</v>
+        <v>57.2</v>
       </c>
       <c r="Q58" t="n">
         <v>1</v>
@@ -4475,7 +4475,7 @@
         <v>9.7761</v>
       </c>
       <c r="P59" t="n">
-        <v>56.5</v>
+        <v>57.2</v>
       </c>
       <c r="Q59" t="n">
         <v>1</v>
@@ -4484,7 +4484,7 @@
         <v>1</v>
       </c>
       <c r="S59" t="n">
-        <v>56.5</v>
+        <v>57.2</v>
       </c>
       <c r="T59" t="n">
         <v>6.5</v>
@@ -4539,7 +4539,7 @@
         <v>15.7132</v>
       </c>
       <c r="P60" t="n">
-        <v>56.5</v>
+        <v>57.2</v>
       </c>
       <c r="Q60" t="n">
         <v>1</v>
@@ -4548,7 +4548,7 @@
         <v>1</v>
       </c>
       <c r="S60" t="n">
-        <v>56.5</v>
+        <v>57.2</v>
       </c>
       <c r="T60" t="n">
         <v>6.4632</v>
@@ -4603,7 +4603,7 @@
         <v>13.9762</v>
       </c>
       <c r="P61" t="n">
-        <v>56.5</v>
+        <v>57.2</v>
       </c>
       <c r="Q61" t="n">
         <v>1</v>
@@ -4612,7 +4612,7 @@
         <v>1</v>
       </c>
       <c r="S61" t="n">
-        <v>56.5</v>
+        <v>57.2</v>
       </c>
       <c r="T61" t="n">
         <v>5.5153</v>
@@ -4665,10 +4665,10 @@
       </c>
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="n">
-        <v>41</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="Q62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R62" t="n">
         <v>0</v>
@@ -4729,10 +4729,10 @@
         <v>9.8222</v>
       </c>
       <c r="P63" t="n">
-        <v>41</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="Q63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R63" t="n">
         <v>0</v>
@@ -4793,10 +4793,10 @@
         <v>8.5106</v>
       </c>
       <c r="P64" t="n">
-        <v>41</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="Q64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R64" t="n">
         <v>0</v>
@@ -4857,16 +4857,16 @@
         <v>18.1992</v>
       </c>
       <c r="P65" t="n">
-        <v>41</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="Q65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R65" t="n">
         <v>1</v>
       </c>
       <c r="S65" t="n">
-        <v>41</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="T65" t="n">
         <v>6.5</v>
@@ -4921,16 +4921,16 @@
         <v>27.6716</v>
       </c>
       <c r="P66" t="n">
-        <v>41</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="Q66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R66" t="n">
         <v>1</v>
       </c>
       <c r="S66" t="n">
-        <v>41</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="T66" t="n">
         <v>6.4632</v>
@@ -4985,16 +4985,16 @@
         <v>18.2322</v>
       </c>
       <c r="P67" t="n">
-        <v>41</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="Q67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R67" t="n">
         <v>1</v>
       </c>
       <c r="S67" t="n">
-        <v>41</v>
+        <v>65.40000000000001</v>
       </c>
       <c r="T67" t="n">
         <v>5.5153</v>
@@ -5811,7 +5811,7 @@
       </c>
       <c r="O80" t="inlineStr"/>
       <c r="P80" t="n">
-        <v>74</v>
+        <v>75.5</v>
       </c>
       <c r="Q80" t="n">
         <v>1</v>
@@ -5875,7 +5875,7 @@
         <v>-3.0321</v>
       </c>
       <c r="P81" t="n">
-        <v>74</v>
+        <v>75.5</v>
       </c>
       <c r="Q81" t="n">
         <v>1</v>
@@ -5939,7 +5939,7 @@
         <v>5.5092</v>
       </c>
       <c r="P82" t="n">
-        <v>74</v>
+        <v>75.5</v>
       </c>
       <c r="Q82" t="n">
         <v>1</v>
@@ -6003,7 +6003,7 @@
         <v>8.2979</v>
       </c>
       <c r="P83" t="n">
-        <v>74</v>
+        <v>75.5</v>
       </c>
       <c r="Q83" t="n">
         <v>1</v>
@@ -6012,7 +6012,7 @@
         <v>1</v>
       </c>
       <c r="S83" t="n">
-        <v>74</v>
+        <v>75.5</v>
       </c>
       <c r="T83" t="n">
         <v>6.5</v>
@@ -6067,7 +6067,7 @@
         <v>7.1459</v>
       </c>
       <c r="P84" t="n">
-        <v>74</v>
+        <v>75.5</v>
       </c>
       <c r="Q84" t="n">
         <v>1</v>
@@ -6076,7 +6076,7 @@
         <v>1</v>
       </c>
       <c r="S84" t="n">
-        <v>74</v>
+        <v>75.5</v>
       </c>
       <c r="T84" t="n">
         <v>6.4632</v>
@@ -6131,7 +6131,7 @@
         <v>7.3122</v>
       </c>
       <c r="P85" t="n">
-        <v>74</v>
+        <v>75.5</v>
       </c>
       <c r="Q85" t="n">
         <v>1</v>
@@ -6140,7 +6140,7 @@
         <v>1</v>
       </c>
       <c r="S85" t="n">
-        <v>74</v>
+        <v>75.5</v>
       </c>
       <c r="T85" t="n">
         <v>5.5153</v>
@@ -6193,7 +6193,7 @@
       </c>
       <c r="O86" t="inlineStr"/>
       <c r="P86" t="n">
-        <v>68.5</v>
+        <v>77</v>
       </c>
       <c r="Q86" t="n">
         <v>1</v>
@@ -6257,7 +6257,7 @@
         <v>21.9585</v>
       </c>
       <c r="P87" t="n">
-        <v>68.5</v>
+        <v>77</v>
       </c>
       <c r="Q87" t="n">
         <v>1</v>
@@ -6321,7 +6321,7 @@
         <v>26.3758</v>
       </c>
       <c r="P88" t="n">
-        <v>68.5</v>
+        <v>77</v>
       </c>
       <c r="Q88" t="n">
         <v>1</v>
@@ -6385,7 +6385,7 @@
         <v>19.2817</v>
       </c>
       <c r="P89" t="n">
-        <v>68.5</v>
+        <v>77</v>
       </c>
       <c r="Q89" t="n">
         <v>1</v>
@@ -6394,7 +6394,7 @@
         <v>1</v>
       </c>
       <c r="S89" t="n">
-        <v>68.5</v>
+        <v>77</v>
       </c>
       <c r="T89" t="n">
         <v>6.5</v>
@@ -6449,7 +6449,7 @@
         <v>12.5766</v>
       </c>
       <c r="P90" t="n">
-        <v>68.5</v>
+        <v>77</v>
       </c>
       <c r="Q90" t="n">
         <v>1</v>
@@ -6458,7 +6458,7 @@
         <v>1</v>
       </c>
       <c r="S90" t="n">
-        <v>68.5</v>
+        <v>77</v>
       </c>
       <c r="T90" t="n">
         <v>6.4632</v>
@@ -6513,7 +6513,7 @@
         <v>14.9036</v>
       </c>
       <c r="P91" t="n">
-        <v>68.5</v>
+        <v>77</v>
       </c>
       <c r="Q91" t="n">
         <v>1</v>
@@ -6522,7 +6522,7 @@
         <v>1</v>
       </c>
       <c r="S91" t="n">
-        <v>68.5</v>
+        <v>77</v>
       </c>
       <c r="T91" t="n">
         <v>5.5153</v>
@@ -6575,7 +6575,7 @@
       </c>
       <c r="O92" t="inlineStr"/>
       <c r="P92" t="n">
-        <v>30.5</v>
+        <v>25.6</v>
       </c>
       <c r="Q92" t="n">
         <v>0</v>
@@ -6639,7 +6639,7 @@
         <v>7.9938</v>
       </c>
       <c r="P93" t="n">
-        <v>30.5</v>
+        <v>25.6</v>
       </c>
       <c r="Q93" t="n">
         <v>0</v>
@@ -6703,7 +6703,7 @@
         <v>37.9854</v>
       </c>
       <c r="P94" t="n">
-        <v>30.5</v>
+        <v>25.6</v>
       </c>
       <c r="Q94" t="n">
         <v>0</v>
@@ -6767,7 +6767,7 @@
         <v>19.1446</v>
       </c>
       <c r="P95" t="n">
-        <v>30.5</v>
+        <v>25.6</v>
       </c>
       <c r="Q95" t="n">
         <v>0</v>
@@ -6776,7 +6776,7 @@
         <v>1</v>
       </c>
       <c r="S95" t="n">
-        <v>30.5</v>
+        <v>25.6</v>
       </c>
       <c r="T95" t="n">
         <v>6.5</v>
@@ -6831,7 +6831,7 @@
         <v>15.739</v>
       </c>
       <c r="P96" t="n">
-        <v>30.5</v>
+        <v>25.6</v>
       </c>
       <c r="Q96" t="n">
         <v>0</v>
@@ -6840,7 +6840,7 @@
         <v>1</v>
       </c>
       <c r="S96" t="n">
-        <v>30.5</v>
+        <v>25.6</v>
       </c>
       <c r="T96" t="n">
         <v>6.4632</v>
@@ -6895,7 +6895,7 @@
         <v>13.0905</v>
       </c>
       <c r="P97" t="n">
-        <v>30.5</v>
+        <v>25.6</v>
       </c>
       <c r="Q97" t="n">
         <v>0</v>
@@ -6904,7 +6904,7 @@
         <v>1</v>
       </c>
       <c r="S97" t="n">
-        <v>30.5</v>
+        <v>25.6</v>
       </c>
       <c r="T97" t="n">
         <v>5.5153</v>
@@ -7923,16 +7923,16 @@
         <v>48</v>
       </c>
       <c r="D4" t="n">
-        <v>51.04</v>
+        <v>51.38</v>
       </c>
       <c r="E4" t="n">
-        <v>15.43</v>
+        <v>16.09</v>
       </c>
       <c r="F4" t="n">
         <v>23</v>
       </c>
       <c r="G4" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5">
@@ -7950,16 +7950,16 @@
         <v>48</v>
       </c>
       <c r="D5" t="n">
-        <v>51.04</v>
+        <v>51.38</v>
       </c>
       <c r="E5" t="n">
-        <v>15.43</v>
+        <v>16.09</v>
       </c>
       <c r="F5" t="n">
         <v>23</v>
       </c>
       <c r="G5" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6">
@@ -8320,24 +8320,20 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.0294</v>
+        <v>0.0063</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0151</v>
+        <v>0.0173</v>
       </c>
       <c r="E2" t="n">
-        <v>0.067</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
+        <v>0.696</v>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>-0.0022</v>
+        <v>-0.0344</v>
       </c>
       <c r="H2" t="n">
-        <v>0.061</v>
+        <v>0.0471</v>
       </c>
       <c r="I2" t="n">
         <v>96</v>
@@ -8346,10 +8342,10 @@
         <v>16</v>
       </c>
       <c r="K2" t="n">
-        <v>0.866</v>
+        <v>0.846</v>
       </c>
       <c r="L2" t="n">
-        <v>0.216</v>
+        <v>0.103</v>
       </c>
     </row>
     <row r="3">
@@ -8364,24 +8360,20 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.0312</v>
+        <v>0.0031</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0168</v>
+        <v>0.019</v>
       </c>
       <c r="E3" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>**</t>
-        </is>
-      </c>
+        <v>0.888</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>0.0022</v>
+        <v>-0.033</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0602</v>
+        <v>0.0391</v>
       </c>
       <c r="I3" t="n">
         <v>96</v>
@@ -8390,10 +8382,10 @@
         <v>16</v>
       </c>
       <c r="K3" t="n">
-        <v>0.856</v>
+        <v>0.834</v>
       </c>
       <c r="L3" t="n">
-        <v>0.137</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="4">
@@ -8408,24 +8400,20 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.0331</v>
+        <v>0.01</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0144</v>
+        <v>0.0164</v>
       </c>
       <c r="E4" t="n">
-        <v>0.027</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>**</t>
-        </is>
-      </c>
+        <v>0.538</v>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>0.0039</v>
+        <v>-0.0281</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0624</v>
+        <v>0.0481</v>
       </c>
       <c r="I4" t="n">
         <v>95</v>
@@ -8434,10 +8422,10 @@
         <v>16</v>
       </c>
       <c r="K4" t="n">
-        <v>0.903</v>
+        <v>0.879</v>
       </c>
       <c r="L4" t="n">
-        <v>0.289</v>
+        <v>0.117</v>
       </c>
     </row>
     <row r="5">
@@ -8452,24 +8440,20 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.0304</v>
+        <v>0.0156</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0119</v>
+        <v>0.014</v>
       </c>
       <c r="E5" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>**</t>
-        </is>
-      </c>
+        <v>0.287</v>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>0.0056</v>
+        <v>-0.0191</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0551</v>
+        <v>0.0503</v>
       </c>
       <c r="I5" t="n">
         <v>80</v>
@@ -8478,10 +8462,10 @@
         <v>16</v>
       </c>
       <c r="K5" t="n">
-        <v>0.923</v>
+        <v>0.909</v>
       </c>
       <c r="L5" t="n">
-        <v>0.327</v>
+        <v>0.204</v>
       </c>
     </row>
     <row r="6">
@@ -8496,24 +8480,20 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.029</v>
+        <v>0.0069</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0152</v>
+        <v>0.0177</v>
       </c>
       <c r="E6" t="n">
-        <v>0.07199999999999999</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
+        <v>0.6860000000000001</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
-        <v>-0.0025</v>
+        <v>-0.0323</v>
       </c>
       <c r="H6" t="n">
-        <v>0.0604</v>
+        <v>0.046</v>
       </c>
       <c r="I6" t="n">
         <v>80</v>
@@ -8522,10 +8502,10 @@
         <v>16</v>
       </c>
       <c r="K6" t="n">
-        <v>0.839</v>
+        <v>0.819</v>
       </c>
       <c r="L6" t="n">
-        <v>0.172</v>
+        <v>0.067</v>
       </c>
     </row>
     <row r="7">
@@ -8540,24 +8520,24 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.0162</v>
+        <v>0.0212</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0103</v>
+        <v>0.01</v>
       </c>
       <c r="E7" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.037</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>*</t>
+          <t>**</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>-0.0012</v>
+        <v>0.0008</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0337</v>
+        <v>0.0416</v>
       </c>
       <c r="I7" t="n">
         <v>96</v>
@@ -8566,10 +8546,10 @@
         <v>16</v>
       </c>
       <c r="K7" t="n">
-        <v>0.866</v>
+        <v>0.847</v>
       </c>
       <c r="L7" t="n">
-        <v>0.228</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="8">
@@ -8584,20 +8564,20 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.4585</v>
+        <v>0.1837</v>
       </c>
       <c r="D8" t="n">
-        <v>0.4365</v>
+        <v>0.4303</v>
       </c>
       <c r="E8" t="n">
-        <v>0.27</v>
+        <v>0.661</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
-        <v>-0.3499</v>
+        <v>-0.6116</v>
       </c>
       <c r="H8" t="n">
-        <v>1.2669</v>
+        <v>0.979</v>
       </c>
       <c r="I8" t="n">
         <v>96</v>
@@ -8606,10 +8586,10 @@
         <v>16</v>
       </c>
       <c r="K8" t="n">
-        <v>0.851</v>
+        <v>0.846</v>
       </c>
       <c r="L8" t="n">
-        <v>0.127</v>
+        <v>0.102</v>
       </c>
     </row>
     <row r="9">
@@ -8624,20 +8604,20 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.0112</v>
+        <v>-0.0176</v>
       </c>
       <c r="D9" t="n">
-        <v>0.0203</v>
+        <v>0.0195</v>
       </c>
       <c r="E9" t="n">
-        <v>0.622</v>
+        <v>0.307</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>-0.0213</v>
+        <v>-0.0474</v>
       </c>
       <c r="H9" t="n">
-        <v>0.0437</v>
+        <v>0.0122</v>
       </c>
       <c r="I9" t="n">
         <v>48</v>
@@ -8646,10 +8626,10 @@
         <v>16</v>
       </c>
       <c r="K9" t="n">
-        <v>0.767</v>
+        <v>0.774</v>
       </c>
       <c r="L9" t="n">
-        <v>0.018</v>
+        <v>0.049</v>
       </c>
     </row>
     <row r="10">
@@ -8664,20 +8644,20 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>-0.06370000000000001</v>
+        <v>0.2505</v>
       </c>
       <c r="D10" t="n">
-        <v>0.267</v>
+        <v>0.2722</v>
       </c>
       <c r="E10" t="n">
-        <v>0.758</v>
+        <v>0.365</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
-        <v>-0.5361</v>
+        <v>-0.1847</v>
       </c>
       <c r="H10" t="n">
-        <v>0.4088</v>
+        <v>0.6857</v>
       </c>
       <c r="I10" t="n">
         <v>80</v>
@@ -8686,10 +8666,10 @@
         <v>16</v>
       </c>
       <c r="K10" t="n">
-        <v>0.274</v>
+        <v>0.305</v>
       </c>
       <c r="L10" t="n">
-        <v>0.059</v>
+        <v>0.099</v>
       </c>
     </row>
   </sheetData>
@@ -8780,20 +8760,20 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-0.0024</v>
+        <v>0.0274</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0234</v>
+        <v>0.0221</v>
       </c>
       <c r="E2" t="n">
-        <v>0.9</v>
+        <v>0.167</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
-        <v>-0.044</v>
+        <v>-0.011</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0392</v>
+        <v>0.0658</v>
       </c>
       <c r="I2" t="n">
         <v>96</v>
@@ -8802,10 +8782,10 @@
         <v>16</v>
       </c>
       <c r="K2" t="n">
-        <v>0.863</v>
+        <v>0.845</v>
       </c>
       <c r="L2" t="n">
-        <v>0.241</v>
+        <v>0.146</v>
       </c>
     </row>
     <row r="3">
@@ -8820,24 +8800,20 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>-0.0192</v>
+        <v>0.0064</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0126</v>
+        <v>0.0144</v>
       </c>
       <c r="E3" t="n">
-        <v>0.094</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>*</t>
-        </is>
-      </c>
+        <v>0.745</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="n">
-        <v>-0.0408</v>
+        <v>-0.0193</v>
       </c>
       <c r="H3" t="n">
-        <v>0.0025</v>
+        <v>0.0321</v>
       </c>
       <c r="I3" t="n">
         <v>96</v>
@@ -8846,10 +8822,10 @@
         <v>16</v>
       </c>
       <c r="K3" t="n">
-        <v>0.863</v>
+        <v>0.845</v>
       </c>
       <c r="L3" t="n">
-        <v>0.241</v>
+        <v>0.146</v>
       </c>
     </row>
     <row r="4">
@@ -8864,24 +8840,20 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.0245</v>
+        <v>0.0155</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0119</v>
+        <v>0.0129</v>
       </c>
       <c r="E4" t="n">
-        <v>0.012</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>**</t>
-        </is>
-      </c>
+        <v>0.268</v>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="n">
-        <v>0.0045</v>
+        <v>-0.0083</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0445</v>
+        <v>0.0394</v>
       </c>
       <c r="I4" t="n">
         <v>96</v>
@@ -8890,10 +8862,10 @@
         <v>16</v>
       </c>
       <c r="K4" t="n">
-        <v>0.863</v>
+        <v>0.845</v>
       </c>
       <c r="L4" t="n">
-        <v>0.241</v>
+        <v>0.146</v>
       </c>
     </row>
     <row r="5">
@@ -8908,24 +8880,20 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.0281</v>
+        <v>0.0171</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0137</v>
+        <v>0.0147</v>
       </c>
       <c r="E5" t="n">
-        <v>0.015</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>**</t>
-        </is>
-      </c>
+        <v>0.278</v>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="n">
-        <v>0.0037</v>
+        <v>-0.0131</v>
       </c>
       <c r="H5" t="n">
-        <v>0.0526</v>
+        <v>0.0473</v>
       </c>
       <c r="I5" t="n">
         <v>96</v>
@@ -8934,10 +8902,10 @@
         <v>16</v>
       </c>
       <c r="K5" t="n">
-        <v>0.863</v>
+        <v>0.845</v>
       </c>
       <c r="L5" t="n">
-        <v>0.241</v>
+        <v>0.146</v>
       </c>
     </row>
     <row r="6">
@@ -8952,20 +8920,24 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.0157</v>
+        <v>0.0203</v>
       </c>
       <c r="D6" t="n">
-        <v>0.0102</v>
+        <v>0.0097</v>
       </c>
       <c r="E6" t="n">
-        <v>0.108</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
+        <v>0.063</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
       <c r="G6" t="n">
-        <v>-0.0019</v>
+        <v>-0.0008</v>
       </c>
       <c r="H6" t="n">
-        <v>0.0332</v>
+        <v>0.0414</v>
       </c>
       <c r="I6" t="n">
         <v>96</v>
@@ -8974,10 +8946,10 @@
         <v>16</v>
       </c>
       <c r="K6" t="n">
-        <v>0.863</v>
+        <v>0.845</v>
       </c>
       <c r="L6" t="n">
-        <v>0.241</v>
+        <v>0.146</v>
       </c>
     </row>
   </sheetData>
@@ -9023,13 +8995,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.029</v>
+        <v>0.0062</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0151</v>
+        <v>0.0175</v>
       </c>
       <c r="D2" t="n">
-        <v>0.0703</v>
+        <v>0.7074</v>
       </c>
     </row>
     <row r="3">
@@ -9039,13 +9011,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.0169</v>
+        <v>0.0198</v>
       </c>
       <c r="C3" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0077</v>
       </c>
       <c r="D3" t="n">
-        <v>0.0983</v>
+        <v>0.0233</v>
       </c>
     </row>
     <row r="4">
@@ -9055,13 +9027,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.0336</v>
+        <v>0.0035</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0174</v>
+        <v>0.0249</v>
       </c>
       <c r="D4" t="n">
-        <v>0.0917</v>
+        <v>0.8693</v>
       </c>
     </row>
     <row r="5">
@@ -9071,13 +9043,13 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0289</v>
+        <v>0.0057</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0156</v>
+        <v>0.0175</v>
       </c>
       <c r="D5" t="n">
-        <v>0.0794</v>
+        <v>0.7369</v>
       </c>
     </row>
     <row r="6">
@@ -9087,13 +9059,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.0295</v>
+        <v>0.0074</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0152</v>
+        <v>0.0168</v>
       </c>
       <c r="D6" t="n">
-        <v>0.06909999999999999</v>
+        <v>0.6427</v>
       </c>
     </row>
     <row r="7">
@@ -9103,13 +9075,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.0311</v>
+        <v>0.0075</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0152</v>
+        <v>0.0171</v>
       </c>
       <c r="D7" t="n">
-        <v>0.0623</v>
+        <v>0.6395999999999999</v>
       </c>
     </row>
     <row r="8">
@@ -9119,13 +9091,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.0302</v>
+        <v>0.007</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0156</v>
+        <v>0.017</v>
       </c>
       <c r="D8" t="n">
-        <v>0.0704</v>
+        <v>0.6604</v>
       </c>
     </row>
     <row r="9">
@@ -9135,13 +9107,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.03</v>
+        <v>0.0067</v>
       </c>
       <c r="C9" t="n">
-        <v>0.0151</v>
+        <v>0.0173</v>
       </c>
       <c r="D9" t="n">
-        <v>0.06320000000000001</v>
+        <v>0.6816</v>
       </c>
     </row>
     <row r="10">
@@ -9151,13 +9123,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.0372</v>
+        <v>0.0073</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0175</v>
+        <v>0.0194</v>
       </c>
       <c r="D10" t="n">
-        <v>0.057</v>
+        <v>0.679</v>
       </c>
     </row>
     <row r="11">
@@ -9167,13 +9139,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.0305</v>
+        <v>0.0072</v>
       </c>
       <c r="C11" t="n">
-        <v>0.015</v>
+        <v>0.0171</v>
       </c>
       <c r="D11" t="n">
-        <v>0.0567</v>
+        <v>0.6532</v>
       </c>
     </row>
     <row r="12">
@@ -9183,13 +9155,13 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.0302</v>
+        <v>0.0064</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0159</v>
+        <v>0.018</v>
       </c>
       <c r="D12" t="n">
-        <v>0.0675</v>
+        <v>0.711</v>
       </c>
     </row>
     <row r="13">
@@ -9199,13 +9171,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.0306</v>
+        <v>0.0069</v>
       </c>
       <c r="C13" t="n">
-        <v>0.0168</v>
+        <v>0.0178</v>
       </c>
       <c r="D13" t="n">
-        <v>0.0687</v>
+        <v>0.6747</v>
       </c>
     </row>
     <row r="14">
@@ -9215,13 +9187,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.0323</v>
+        <v>0.0097</v>
       </c>
       <c r="C14" t="n">
-        <v>0.0154</v>
+        <v>0.0156</v>
       </c>
       <c r="D14" t="n">
-        <v>0.0476</v>
+        <v>0.518</v>
       </c>
     </row>
     <row r="15">
@@ -9231,13 +9203,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.0276</v>
+        <v>0.0003</v>
       </c>
       <c r="C15" t="n">
-        <v>0.018</v>
+        <v>0.0209</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1493</v>
+        <v>0.9861</v>
       </c>
     </row>
     <row r="16">
@@ -9247,13 +9219,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.0287</v>
+        <v>0.0021</v>
       </c>
       <c r="C16" t="n">
-        <v>0.0177</v>
+        <v>0.0189</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1382</v>
+        <v>0.9077</v>
       </c>
     </row>
     <row r="17">
@@ -9263,13 +9235,13 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.0246</v>
+        <v>-0.003</v>
       </c>
       <c r="C17" t="n">
-        <v>0.0143</v>
+        <v>0.0203</v>
       </c>
       <c r="D17" t="n">
-        <v>0.1393</v>
+        <v>0.9211</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Apply report template layout; add certificate, executive summary, rationale, theoretical framework, ANOVA/model summary, diagnostics and inference-sensitivity tables
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QUxicXQrqdyqQxohnFLPv8
</commit_message>
<xml_diff>
--- a/Dissertation_Data.xlsx
+++ b/Dissertation_Data.xlsx
@@ -21,6 +21,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results_Firm" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results_COF_Event" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results_BankShare_Event" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results_ModelSummary" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results_Inference" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RBI_Descriptives" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RBI_Correlation" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,9 +33,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -62,9 +65,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -577,10 +581,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>All regression results reported in the dissertation</t>
+          <t>All regression results reported in the dissertation (Results_ModelSummary: R2, ANOVA, coefficients and diagnostics of Models 1-2; Results_Inference: p-values under alternative standard errors)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
+        <is>
+          <t>This study</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>RBI_Descriptives / RBI_Correlation</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Descriptive statistics and correlation matrix of monthly growth rates (Tables 4.4-4.5)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t>This study</t>
         </is>
@@ -671,8 +692,6 @@
       <c r="G2" t="n">
         <v>-7.9421</v>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -680,8 +699,6 @@
           <t>H1 panel DiD (Driscoll-Kraay)</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
         <v>0.2457</v>
       </c>
@@ -691,7 +708,6 @@
       <c r="F3" t="n">
         <v>229</v>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="n">
         <v>-0.6624</v>
       </c>
@@ -723,8 +739,6 @@
       <c r="G4" t="n">
         <v>5.4019</v>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -750,8 +764,6 @@
       <c r="G5" t="n">
         <v>-11.9439</v>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -777,8 +789,6 @@
       <c r="G6" t="n">
         <v>3.2534</v>
       </c>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -804,8 +814,6 @@
       <c r="G7" t="n">
         <v>-16.9313</v>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -831,8 +839,6 @@
       <c r="G8" t="n">
         <v>-7.5556</v>
       </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -858,8 +864,6 @@
       <c r="G9" t="n">
         <v>11.4255</v>
       </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1126,7 +1130,6 @@
       <c r="F2" t="n">
         <v>16</v>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1149,7 +1152,6 @@
       <c r="F3" t="n">
         <v>16</v>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1172,7 +1174,6 @@
       <c r="F4" t="n">
         <v>15</v>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1183,13 +1184,9 @@
       <c r="B5" t="n">
         <v>-1.618392784713566</v>
       </c>
-      <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
         <v>0.5653282664133207</v>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1209,7 +1206,6 @@
       <c r="E6" t="n">
         <v>171</v>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
         <v>9</v>
       </c>
@@ -1388,7 +1384,6 @@
       <c r="E7" t="n">
         <v>0</v>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1696,7 +1691,6 @@
       <c r="E7" t="n">
         <v>0</v>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1828,6 +1822,1353 @@
       </c>
       <c r="F13" t="n">
         <v>0.1185559277963898</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Z3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>r2</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>adj_r2</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>f</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>f_p</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>ss_model</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>ss_resid</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>df_model</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>df_resid</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>const</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>const_se</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>const_p</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>delta</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>delta_se</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>delta_p</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>jb</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>jb_p</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>skew</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>kurt</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>dw</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>lb12</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>lb12_p</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>bp</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>bp_p</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>vif</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>46</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.04032911121147364</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.01851840919355263</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1.849051496753142</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.1808212926435636</v>
+      </c>
+      <c r="G2" t="n">
+        <v>4.266090982701172</v>
+      </c>
+      <c r="H2" t="n">
+        <v>101.5158331547061</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>44</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.6732466688588704</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0.1701283897561112</v>
+      </c>
+      <c r="M2" t="n">
+        <v>7.58061971222136e-05</v>
+      </c>
+      <c r="N2" t="n">
+        <v>-0.6618429781209935</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.2155612086957849</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.002138259200481926</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>2.267582475777944</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.3218108791268169</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.438273227430507</v>
+      </c>
+      <c r="T2" t="n">
+        <v>3.644013060094378</v>
+      </c>
+      <c r="U2" t="n">
+        <v>2.214387180630642</v>
+      </c>
+      <c r="V2" t="n">
+        <v>19.61158395988117</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0.07479954999683637</v>
+      </c>
+      <c r="X2" t="n">
+        <v>3.153195277235476</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0.07577844036809317</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>45</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.04146083876401463</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.01916923036317775</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.859930338739404</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.179729933009793</v>
+      </c>
+      <c r="G3" t="n">
+        <v>9.554467311956103</v>
+      </c>
+      <c r="H3" t="n">
+        <v>220.8911193376021</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>43</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.8926193468508969</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0.4288328828267325</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.03738737492155869</v>
+      </c>
+      <c r="N3" t="n">
+        <v>-0.9953243560871659</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.5049012182476404</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.04868672217907708</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>3.413223841842864</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.1814796194849206</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.6609938005408814</v>
+      </c>
+      <c r="T3" t="n">
+        <v>3.269693959088718</v>
+      </c>
+      <c r="U3" t="n">
+        <v>2.007041133860301</v>
+      </c>
+      <c r="V3" t="n">
+        <v>8.175037173169034</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.771306551651752</v>
+      </c>
+      <c r="X3" t="n">
+        <v>1.467807784636374</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0.225691894644438</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>delta_H1</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>p_H1</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>delta_H2</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>p_H2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Classical OLS</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>-0.662</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.181</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-0.995</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>White (HC1)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>-0.662</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.089</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-0.995</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.122</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Newey-West, 1 lag</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>-0.662</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.076</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-0.995</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.104</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Newey-West, 3 lags (rule of thumb)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>-0.662</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-0.995</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.08599999999999999</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Newey-West, 6 lags (main)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>-0.662</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-0.995</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.049</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Newey-West, 12 lags</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>-0.662</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-0.995</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.026</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Month dummies, classical OLS</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>-0.6909999999999999</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.107</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-1.18</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.065</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Month dummies, White (HC1)</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>-0.6909999999999999</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.102</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-1.18</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.043</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Month dummies, Newey-West 3 lags</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>-0.6909999999999999</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-1.18</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.012</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Moving-block bootstrap (block 3)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>-0.662</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.106</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-0.995</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Month dummies, moving-block bootstrap</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>-0.6909999999999999</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.064</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-1.18</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.047</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Series</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Mean</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>SD</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Credit cards</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Pre-policy</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D2" t="n">
+        <v>1.944</v>
+      </c>
+      <c r="E2" t="n">
+        <v>3.07</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-7.575</v>
+      </c>
+      <c r="G2" t="n">
+        <v>7.983</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Credit cards</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Post-policy</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>14</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1.265</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-1.737</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3.464</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Other personal loans</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Pre-policy</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>31</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1.194</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-0.795</v>
+      </c>
+      <c r="G4" t="n">
+        <v>4.038</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Other personal loans</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Post-policy</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>14</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.838</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.867</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-0.775</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2.612</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Pre-policy</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>30</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.157</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.859</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-0.43</v>
+      </c>
+      <c r="G6" t="n">
+        <v>3.488</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Post-policy</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>14</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.928</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.436</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.412</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.771</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Vehicle loans</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Pre-policy</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>31</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1.217</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1.359</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-1.61</v>
+      </c>
+      <c r="G8" t="n">
+        <v>4.137</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Vehicle loans</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Post-policy</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>14</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.8159999999999999</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.753</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-0.446</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2.639</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Pre-policy</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>31</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1.129</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1.224</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-0.861</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4.218</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Post-policy</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>14</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.8120000000000001</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-0.214</v>
+      </c>
+      <c r="G11" t="n">
+        <v>2.564</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>NBFCs ex-HFC</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Pre-policy</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>30</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1.956</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3.143</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-4.379</v>
+      </c>
+      <c r="G12" t="n">
+        <v>9.279999999999999</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>NBFCs ex-HFC</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Post-policy</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>14</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.761</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1.927</v>
+      </c>
+      <c r="F13" t="n">
+        <v>-2.876</v>
+      </c>
+      <c r="G13" t="n">
+        <v>3.814</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>HFCs</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pre-policy</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>30</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.588</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2.431</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-3.453</v>
+      </c>
+      <c r="G14" t="n">
+        <v>7.223</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>HFCs</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Post-policy</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>14</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2.468</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-2.586</v>
+      </c>
+      <c r="G15" t="n">
+        <v>7.388</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Non-food credit</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Pre-policy</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>30</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1.096</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-0.9340000000000001</v>
+      </c>
+      <c r="G16" t="n">
+        <v>3.665</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Non-food credit</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Post-policy</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>14</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.864</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.772</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-0.546</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2.385</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Credit cards</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Other personal loans</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Vehicle loans</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>NBFCs ex-HFC</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>HFCs</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Non-food credit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Credit cards</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Other personal loans</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.53</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Housing</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Vehicle loans</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.27</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NBFCs ex-HFC</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>HFCs</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Non-food credit</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1952,7 +3293,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" s="2" t="n">
         <v>43483</v>
       </c>
       <c r="B2" t="n">
@@ -1985,19 +3326,9 @@
       <c r="K2" t="n">
         <v>455555.11</v>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" s="2" t="n">
         <v>43511</v>
       </c>
       <c r="B3" t="n">
@@ -2062,7 +3393,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" s="2" t="n">
         <v>43553</v>
       </c>
       <c r="B4" t="n">
@@ -2127,7 +3458,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="2" t="n">
         <v>43581</v>
       </c>
       <c r="B5" t="n">
@@ -2192,7 +3523,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="2" t="n">
         <v>43609</v>
       </c>
       <c r="B6" t="n">
@@ -2257,7 +3588,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
+      <c r="A7" s="2" t="n">
         <v>43637</v>
       </c>
       <c r="B7" t="n">
@@ -2322,7 +3653,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="2" t="n">
         <v>43665</v>
       </c>
       <c r="B8" t="n">
@@ -2387,7 +3718,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
+      <c r="A9" s="2" t="n">
         <v>43707</v>
       </c>
       <c r="B9" t="n">
@@ -2452,7 +3783,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
+      <c r="A10" s="2" t="n">
         <v>43735</v>
       </c>
       <c r="B10" t="n">
@@ -2517,7 +3848,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="A11" s="2" t="n">
         <v>43763</v>
       </c>
       <c r="B11" t="n">
@@ -2582,7 +3913,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="1" t="n">
+      <c r="A12" s="2" t="n">
         <v>43791</v>
       </c>
       <c r="B12" t="n">
@@ -2647,7 +3978,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1" t="n">
+      <c r="A13" s="2" t="n">
         <v>43819</v>
       </c>
       <c r="B13" t="n">
@@ -2712,7 +4043,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n">
+      <c r="A14" s="2" t="n">
         <v>43861</v>
       </c>
       <c r="B14" t="n">
@@ -2777,7 +4108,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="1" t="n">
+      <c r="A15" s="2" t="n">
         <v>43889</v>
       </c>
       <c r="B15" t="n">
@@ -2842,7 +4173,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="n">
+      <c r="A16" s="2" t="n">
         <v>43917</v>
       </c>
       <c r="B16" t="n">
@@ -2907,7 +4238,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="1" t="n">
+      <c r="A17" s="2" t="n">
         <v>43945</v>
       </c>
       <c r="B17" t="n">
@@ -2972,7 +4303,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="n">
+      <c r="A18" s="2" t="n">
         <v>43973</v>
       </c>
       <c r="B18" t="n">
@@ -3037,7 +4368,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n">
+      <c r="A19" s="2" t="n">
         <v>44001</v>
       </c>
       <c r="B19" t="n">
@@ -3102,7 +4433,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1" t="n">
+      <c r="A20" s="2" t="n">
         <v>44043</v>
       </c>
       <c r="B20" t="n">
@@ -3167,7 +4498,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n">
+      <c r="A21" s="2" t="n">
         <v>44071</v>
       </c>
       <c r="B21" t="n">
@@ -3232,7 +4563,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="1" t="n">
+      <c r="A22" s="2" t="n">
         <v>44099</v>
       </c>
       <c r="B22" t="n">
@@ -3297,7 +4628,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="n">
+      <c r="A23" s="2" t="n">
         <v>44127</v>
       </c>
       <c r="B23" t="n">
@@ -3362,7 +4693,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="n">
+      <c r="A24" s="2" t="n">
         <v>44155</v>
       </c>
       <c r="B24" t="n">
@@ -3427,7 +4758,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" s="2" t="n">
         <v>44183</v>
       </c>
       <c r="B25" t="n">
@@ -3492,7 +4823,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1" t="n">
+      <c r="A26" s="2" t="n">
         <v>44225</v>
       </c>
       <c r="B26" t="n">
@@ -3557,7 +4888,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
+      <c r="A27" s="2" t="n">
         <v>44253</v>
       </c>
       <c r="B27" t="n">
@@ -3622,7 +4953,7 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="n">
+      <c r="A28" s="2" t="n">
         <v>44281</v>
       </c>
       <c r="B28" t="n">
@@ -3687,7 +5018,7 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1" t="n">
+      <c r="A29" s="2" t="n">
         <v>44309</v>
       </c>
       <c r="B29" t="n">
@@ -3752,7 +5083,7 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n">
+      <c r="A30" s="2" t="n">
         <v>44337</v>
       </c>
       <c r="B30" t="n">
@@ -3817,7 +5148,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1" t="n">
+      <c r="A31" s="2" t="n">
         <v>44365</v>
       </c>
       <c r="B31" t="n">
@@ -3882,7 +5213,7 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="n">
+      <c r="A32" s="2" t="n">
         <v>44407</v>
       </c>
       <c r="B32" t="n">
@@ -3947,7 +5278,7 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="n">
+      <c r="A33" s="2" t="n">
         <v>44435</v>
       </c>
       <c r="B33" t="n">
@@ -4012,7 +5343,7 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="n">
+      <c r="A34" s="2" t="n">
         <v>44463</v>
       </c>
       <c r="B34" t="n">
@@ -4077,7 +5408,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="n">
+      <c r="A35" s="2" t="n">
         <v>44491</v>
       </c>
       <c r="B35" t="n">
@@ -4142,7 +5473,7 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="A36" s="2" t="n">
         <v>44519</v>
       </c>
       <c r="B36" t="n">
@@ -4207,7 +5538,7 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="n">
+      <c r="A37" s="2" t="n">
         <v>44561</v>
       </c>
       <c r="B37" t="n">
@@ -4272,7 +5603,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="n">
+      <c r="A38" s="2" t="n">
         <v>44589</v>
       </c>
       <c r="B38" t="n">
@@ -4337,7 +5668,7 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="n">
+      <c r="A39" s="2" t="n">
         <v>44617</v>
       </c>
       <c r="B39" t="n">
@@ -4402,7 +5733,7 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="n">
+      <c r="A40" s="2" t="n">
         <v>44645</v>
       </c>
       <c r="B40" t="n">
@@ -4467,7 +5798,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="n">
+      <c r="A41" s="2" t="n">
         <v>44673</v>
       </c>
       <c r="B41" t="n">
@@ -4532,7 +5863,7 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="n">
+      <c r="A42" s="2" t="n">
         <v>44701</v>
       </c>
       <c r="B42" t="n">
@@ -4597,7 +5928,7 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="n">
+      <c r="A43" s="2" t="n">
         <v>44729</v>
       </c>
       <c r="B43" t="n">
@@ -4662,7 +5993,7 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="n">
+      <c r="A44" s="2" t="n">
         <v>44771</v>
       </c>
       <c r="B44" t="n">
@@ -4727,7 +6058,7 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="n">
+      <c r="A45" s="2" t="n">
         <v>44799</v>
       </c>
       <c r="B45" t="n">
@@ -4792,7 +6123,7 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n">
+      <c r="A46" s="2" t="n">
         <v>44827</v>
       </c>
       <c r="B46" t="n">
@@ -4857,7 +6188,7 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="n">
+      <c r="A47" s="2" t="n">
         <v>44855</v>
       </c>
       <c r="B47" t="n">
@@ -4922,7 +6253,7 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n">
+      <c r="A48" s="2" t="n">
         <v>44883</v>
       </c>
       <c r="B48" t="n">
@@ -4987,7 +6318,7 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="n">
+      <c r="A49" s="2" t="n">
         <v>44925</v>
       </c>
       <c r="B49" t="n">
@@ -5052,7 +6383,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1" t="n">
+      <c r="A50" s="2" t="n">
         <v>44953</v>
       </c>
       <c r="B50" t="n">
@@ -5117,7 +6448,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="n">
+      <c r="A51" s="2" t="n">
         <v>44981</v>
       </c>
       <c r="B51" t="n">
@@ -5182,7 +6513,7 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" s="2" t="n">
         <v>45009</v>
       </c>
       <c r="B52" t="n">
@@ -5247,7 +6578,7 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
+      <c r="A53" s="2" t="n">
         <v>45037</v>
       </c>
       <c r="B53" t="n">
@@ -5312,7 +6643,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" s="2" t="n">
         <v>45065</v>
       </c>
       <c r="B54" t="n">
@@ -5377,7 +6708,7 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1" t="n">
+      <c r="A55" s="2" t="n">
         <v>45107</v>
       </c>
       <c r="B55" t="n">
@@ -5442,7 +6773,7 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1" t="n">
+      <c r="A56" s="2" t="n">
         <v>45135</v>
       </c>
       <c r="B56" t="n">
@@ -5475,10 +6806,6 @@
       <c r="K56" t="n">
         <v>1035975.863548</v>
       </c>
-      <c r="L56" t="inlineStr"/>
-      <c r="M56" t="inlineStr"/>
-      <c r="N56" t="inlineStr"/>
-      <c r="O56" t="inlineStr"/>
       <c r="P56" t="n">
         <v>2.047905472771916</v>
       </c>
@@ -5494,10 +6821,9 @@
       <c r="T56" t="n">
         <v>2.135216261553552</v>
       </c>
-      <c r="U56" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" s="1" t="n">
+      <c r="A57" s="2" t="n">
         <v>45163</v>
       </c>
       <c r="B57" t="n">
@@ -5562,7 +6888,7 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="1" t="n">
+      <c r="A58" s="2" t="n">
         <v>45191</v>
       </c>
       <c r="B58" t="n">
@@ -5627,7 +6953,7 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="1" t="n">
+      <c r="A59" s="2" t="n">
         <v>45219</v>
       </c>
       <c r="B59" t="n">
@@ -5692,7 +7018,7 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="1" t="n">
+      <c r="A60" s="2" t="n">
         <v>45247</v>
       </c>
       <c r="B60" t="n">
@@ -5757,7 +7083,7 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="1" t="n">
+      <c r="A61" s="2" t="n">
         <v>45289</v>
       </c>
       <c r="B61" t="n">
@@ -5822,7 +7148,7 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
+      <c r="A62" s="2" t="n">
         <v>45317</v>
       </c>
       <c r="B62" t="n">
@@ -5887,7 +7213,7 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="1" t="n">
+      <c r="A63" s="2" t="n">
         <v>45345</v>
       </c>
       <c r="B63" t="n">
@@ -5952,7 +7278,7 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="1" t="n">
+      <c r="A64" s="2" t="n">
         <v>45373</v>
       </c>
       <c r="B64" t="n">
@@ -6017,7 +7343,7 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="1" t="n">
+      <c r="A65" s="2" t="n">
         <v>45401</v>
       </c>
       <c r="B65" t="n">
@@ -6082,7 +7408,7 @@
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="1" t="n">
+      <c r="A66" s="2" t="n">
         <v>45443</v>
       </c>
       <c r="B66" t="n">
@@ -6147,7 +7473,7 @@
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="1" t="n">
+      <c r="A67" s="2" t="n">
         <v>45471</v>
       </c>
       <c r="B67" t="n">
@@ -6212,7 +7538,7 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="n">
+      <c r="A68" s="2" t="n">
         <v>45499</v>
       </c>
       <c r="B68" t="n">
@@ -6277,7 +7603,7 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
+      <c r="A69" s="2" t="n">
         <v>45527</v>
       </c>
       <c r="B69" t="n">
@@ -6342,7 +7668,7 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" s="2" t="n">
         <v>45555</v>
       </c>
       <c r="B70" t="n">
@@ -6407,7 +7733,7 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="1" t="n">
+      <c r="A71" s="2" t="n">
         <v>45583</v>
       </c>
       <c r="B71" t="n">
@@ -6472,7 +7798,7 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="1" t="n">
+      <c r="A72" s="2" t="n">
         <v>45625</v>
       </c>
       <c r="B72" t="n">
@@ -6537,7 +7863,7 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="1" t="n">
+      <c r="A73" s="2" t="n">
         <v>45653</v>
       </c>
       <c r="B73" t="n">
@@ -6602,7 +7928,7 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="1" t="n">
+      <c r="A74" s="2" t="n">
         <v>45681</v>
       </c>
       <c r="B74" t="n">
@@ -6667,7 +7993,7 @@
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="1" t="n">
+      <c r="A75" s="2" t="n">
         <v>45709</v>
       </c>
       <c r="B75" t="n">
@@ -6732,7 +8058,7 @@
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="1" t="n">
+      <c r="A76" s="2" t="n">
         <v>45737</v>
       </c>
       <c r="B76" t="n">
@@ -6797,7 +8123,7 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="1" t="n">
+      <c r="A77" s="2" t="n">
         <v>45765</v>
       </c>
       <c r="B77" t="n">
@@ -6862,7 +8188,7 @@
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
+      <c r="A78" s="2" t="n">
         <v>45807</v>
       </c>
       <c r="B78" t="n">
@@ -6927,7 +8253,7 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="1" t="n">
+      <c r="A79" s="2" t="n">
         <v>45835</v>
       </c>
       <c r="B79" t="n">
@@ -6992,7 +8318,7 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="1" t="n">
+      <c r="A80" s="2" t="n">
         <v>45863</v>
       </c>
       <c r="B80" t="n">
@@ -7057,7 +8383,7 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="1" t="n">
+      <c r="A81" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="B81" t="n">
@@ -7122,7 +8448,7 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="1" t="n">
+      <c r="A82" s="2" t="n">
         <v>45919</v>
       </c>
       <c r="B82" t="n">
@@ -7187,7 +8513,7 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="1" t="n">
+      <c r="A83" s="2" t="n">
         <v>45961</v>
       </c>
       <c r="B83" t="n">
@@ -7252,7 +8578,7 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="1" t="n">
+      <c r="A84" s="2" t="n">
         <v>45989</v>
       </c>
       <c r="B84" t="n">
@@ -7317,7 +8643,7 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="1" t="n">
+      <c r="A85" s="2" t="n">
         <v>46022</v>
       </c>
       <c r="B85" t="n">
@@ -7382,7 +8708,7 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="1" t="n">
+      <c r="A86" s="2" t="n">
         <v>46053</v>
       </c>
       <c r="B86" t="n">
@@ -7447,7 +8773,7 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
+      <c r="A87" s="2" t="n">
         <v>46081</v>
       </c>
       <c r="B87" t="n">
@@ -7512,7 +8838,7 @@
       </c>
     </row>
     <row r="88">
-      <c r="A88" s="1" t="n">
+      <c r="A88" s="2" t="n">
         <v>46112</v>
       </c>
       <c r="B88" t="n">
@@ -7577,7 +8903,7 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="1" t="n">
+      <c r="A89" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="B89" t="n">
@@ -7642,7 +8968,7 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="1" t="n">
+      <c r="A90" s="2" t="n">
         <v>46173</v>
       </c>
       <c r="B90" t="n">
@@ -7707,7 +9033,7 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="1" t="n">
+      <c r="A91" s="2" t="n">
         <v>46203</v>
       </c>
       <c r="B91" t="n">
@@ -7772,7 +9098,7 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="1" t="n">
+      <c r="A92" s="2" t="n">
         <v>46234</v>
       </c>
       <c r="B92" t="n">
@@ -8162,7 +9488,6 @@
           <t>21-3 / 21-4 p.15</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8188,7 +9513,6 @@
           <t>21-4 p.15</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8214,7 +9538,6 @@
           <t>22-1</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8240,7 +9563,6 @@
           <t>22-2</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8266,7 +9588,6 @@
           <t>22-4 p.14</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -8292,7 +9613,6 @@
           <t>22-4 p.14 / 23-4 p.17</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8348,7 +9668,6 @@
           <t>23-4 p.17</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8374,7 +9693,6 @@
           <t>23-4 p.17</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -8400,7 +9718,6 @@
           <t>23-4 p.17</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8426,7 +9743,6 @@
           <t>24-1 / 24-3</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -8452,7 +9768,6 @@
           <t>24-2 / 24-3</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -8478,7 +9793,6 @@
           <t>24-3 (5-quarter series)</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -8504,7 +9818,6 @@
           <t>24-4 key metrics</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -8530,7 +9843,6 @@
           <t>25-1 / 25-4 p.17</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -8556,7 +9868,6 @@
           <t>25-4 p.17</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -8582,7 +9893,6 @@
           <t>25-4 p.17</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -8638,7 +9948,6 @@
           <t>26-2 (prior-quarter column)</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -8664,7 +9973,6 @@
           <t>26-2 key metrics</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -8690,7 +9998,6 @@
           <t>26-3 / 26-4</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -8716,7 +10023,6 @@
           <t>26-4 key metrics</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">

</xml_diff>

<commit_message>
Remove manual spot-check placeholders and spot-check sample
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QUxicXQrqdyqQxohnFLPv8
</commit_message>
<xml_diff>
--- a/Dissertation_Data.xlsx
+++ b/Dissertation_Data.xlsx
@@ -26,10 +26,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RBI_Descriptives" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RBI_Correlation" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extraction_Recheck" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Manual_Spot_Check" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results_BankShare_Subsamples" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results_EventStudy_H1" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results_EventStudy_H2" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results_BankShare_Subsamples" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results_EventStudy_H1" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results_EventStudy_H2" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4974,7 +4973,6 @@
       <c r="G47" t="b">
         <v>1</v>
       </c>
-      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5008,7 +5006,6 @@
       <c r="G48" t="b">
         <v>1</v>
       </c>
-      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5042,7 +5039,6 @@
       <c r="G49" t="b">
         <v>1</v>
       </c>
-      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5076,7 +5072,6 @@
       <c r="G50" t="b">
         <v>1</v>
       </c>
-      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5110,7 +5105,6 @@
       <c r="G51" t="b">
         <v>1</v>
       </c>
-      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5144,7 +5138,6 @@
       <c r="G52" t="b">
         <v>1</v>
       </c>
-      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5178,7 +5171,6 @@
       <c r="G53" t="b">
         <v>1</v>
       </c>
-      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5212,7 +5204,6 @@
       <c r="G54" t="b">
         <v>1</v>
       </c>
-      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5246,7 +5237,6 @@
       <c r="G55" t="b">
         <v>1</v>
       </c>
-      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5280,7 +5270,6 @@
       <c r="G56" t="b">
         <v>1</v>
       </c>
-      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5314,7 +5303,6 @@
       <c r="G57" t="b">
         <v>1</v>
       </c>
-      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5348,7 +5336,6 @@
       <c r="G58" t="b">
         <v>1</v>
       </c>
-      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5382,7 +5369,6 @@
       <c r="G59" t="b">
         <v>1</v>
       </c>
-      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5416,7 +5402,6 @@
       <c r="G60" t="b">
         <v>1</v>
       </c>
-      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5450,7 +5435,6 @@
       <c r="G61" t="b">
         <v>1</v>
       </c>
-      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5484,7 +5468,6 @@
       <c r="G62" t="b">
         <v>1</v>
       </c>
-      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5518,7 +5501,6 @@
       <c r="G63" t="b">
         <v>1</v>
       </c>
-      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5552,7 +5534,6 @@
       <c r="G64" t="b">
         <v>1</v>
       </c>
-      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5586,7 +5567,6 @@
       <c r="G65" t="b">
         <v>1</v>
       </c>
-      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5620,7 +5600,6 @@
       <c r="G66" t="b">
         <v>1</v>
       </c>
-      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5654,7 +5633,6 @@
       <c r="G67" t="b">
         <v>1</v>
       </c>
-      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5688,7 +5666,6 @@
       <c r="G68" t="b">
         <v>1</v>
       </c>
-      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5722,7 +5699,6 @@
       <c r="G69" t="b">
         <v>1</v>
       </c>
-      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5756,7 +5732,6 @@
       <c r="G70" t="b">
         <v>1</v>
       </c>
-      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5790,7 +5765,6 @@
       <c r="G71" t="b">
         <v>1</v>
       </c>
-      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5824,7 +5798,6 @@
       <c r="G72" t="b">
         <v>1</v>
       </c>
-      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5858,7 +5831,6 @@
       <c r="G73" t="b">
         <v>1</v>
       </c>
-      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5892,7 +5864,6 @@
       <c r="G74" t="b">
         <v>1</v>
       </c>
-      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5926,7 +5897,6 @@
       <c r="G75" t="b">
         <v>1</v>
       </c>
-      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5960,7 +5930,6 @@
       <c r="G76" t="b">
         <v>1</v>
       </c>
-      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5994,7 +5963,6 @@
       <c r="G77" t="b">
         <v>1</v>
       </c>
-      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6028,7 +5996,6 @@
       <c r="G78" t="b">
         <v>1</v>
       </c>
-      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6062,7 +6029,6 @@
       <c r="G79" t="b">
         <v>1</v>
       </c>
-      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6096,7 +6062,6 @@
       <c r="G80" t="b">
         <v>1</v>
       </c>
-      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6130,7 +6095,6 @@
       <c r="G81" t="b">
         <v>1</v>
       </c>
-      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6164,7 +6128,6 @@
       <c r="G82" t="b">
         <v>1</v>
       </c>
-      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6198,7 +6161,6 @@
       <c r="G83" t="b">
         <v>1</v>
       </c>
-      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6232,7 +6194,6 @@
       <c r="G84" t="b">
         <v>1</v>
       </c>
-      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6266,7 +6227,6 @@
       <c r="G85" t="b">
         <v>1</v>
       </c>
-      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6300,7 +6260,6 @@
       <c r="G86" t="b">
         <v>1</v>
       </c>
-      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6334,7 +6293,6 @@
       <c r="G87" t="b">
         <v>1</v>
       </c>
-      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6368,7 +6326,6 @@
       <c r="G88" t="b">
         <v>1</v>
       </c>
-      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6402,7 +6359,6 @@
       <c r="G89" t="b">
         <v>1</v>
       </c>
-      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6436,7 +6392,6 @@
       <c r="G90" t="b">
         <v>1</v>
       </c>
-      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6470,7 +6425,6 @@
       <c r="G91" t="b">
         <v>1</v>
       </c>
-      <c r="H91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6504,7 +6458,6 @@
       <c r="G92" t="b">
         <v>1</v>
       </c>
-      <c r="H92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -6538,7 +6491,6 @@
       <c r="G93" t="b">
         <v>1</v>
       </c>
-      <c r="H93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -6572,7 +6524,6 @@
       <c r="G94" t="b">
         <v>1</v>
       </c>
-      <c r="H94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7434,7 +7385,6 @@
       <c r="G118" t="b">
         <v>1</v>
       </c>
-      <c r="H118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -7468,7 +7418,6 @@
       <c r="G119" t="b">
         <v>1</v>
       </c>
-      <c r="H119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -7502,7 +7451,6 @@
       <c r="G120" t="b">
         <v>1</v>
       </c>
-      <c r="H120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -7536,7 +7484,6 @@
       <c r="G121" t="b">
         <v>1</v>
       </c>
-      <c r="H121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -7570,7 +7517,6 @@
       <c r="G122" t="b">
         <v>1</v>
       </c>
-      <c r="H122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -7604,7 +7550,6 @@
       <c r="G123" t="b">
         <v>1</v>
       </c>
-      <c r="H123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -7638,7 +7583,6 @@
       <c r="G124" t="b">
         <v>1</v>
       </c>
-      <c r="H124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -7672,7 +7616,6 @@
       <c r="G125" t="b">
         <v>1</v>
       </c>
-      <c r="H125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -7706,7 +7649,6 @@
       <c r="G126" t="b">
         <v>1</v>
       </c>
-      <c r="H126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -7740,7 +7682,6 @@
       <c r="G127" t="b">
         <v>1</v>
       </c>
-      <c r="H127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -7774,7 +7715,6 @@
       <c r="G128" t="b">
         <v>1</v>
       </c>
-      <c r="H128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -7808,7 +7748,6 @@
       <c r="G129" t="b">
         <v>1</v>
       </c>
-      <c r="H129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -7842,7 +7781,6 @@
       <c r="G130" t="b">
         <v>1</v>
       </c>
-      <c r="H130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -7876,7 +7814,6 @@
       <c r="G131" t="b">
         <v>1</v>
       </c>
-      <c r="H131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -7910,7 +7847,6 @@
       <c r="G132" t="b">
         <v>1</v>
       </c>
-      <c r="H132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -7944,7 +7880,6 @@
       <c r="G133" t="b">
         <v>1</v>
       </c>
-      <c r="H133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -14674,7 +14609,6 @@
       <c r="G320" t="b">
         <v>0</v>
       </c>
-      <c r="H320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -14708,7 +14642,6 @@
       <c r="G321" t="b">
         <v>0</v>
       </c>
-      <c r="H321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -14742,7 +14675,6 @@
       <c r="G322" t="b">
         <v>0</v>
       </c>
-      <c r="H322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -14776,7 +14708,6 @@
       <c r="G323" t="b">
         <v>0</v>
       </c>
-      <c r="H323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -14810,7 +14741,6 @@
       <c r="G324" t="b">
         <v>0</v>
       </c>
-      <c r="H324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -14844,7 +14774,6 @@
       <c r="G325" t="b">
         <v>0</v>
       </c>
-      <c r="H325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -14878,7 +14807,6 @@
       <c r="G326" t="b">
         <v>0</v>
       </c>
-      <c r="H326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -14912,7 +14840,6 @@
       <c r="G327" t="b">
         <v>0</v>
       </c>
-      <c r="H327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -14946,7 +14873,6 @@
       <c r="G328" t="b">
         <v>0</v>
       </c>
-      <c r="H328" t="inlineStr"/>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -14980,7 +14906,6 @@
       <c r="G329" t="b">
         <v>0</v>
       </c>
-      <c r="H329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -15014,7 +14939,6 @@
       <c r="G330" t="b">
         <v>0</v>
       </c>
-      <c r="H330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -15048,7 +14972,6 @@
       <c r="G331" t="b">
         <v>0</v>
       </c>
-      <c r="H331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -15082,7 +15005,6 @@
       <c r="G332" t="b">
         <v>0</v>
       </c>
-      <c r="H332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -15116,7 +15038,6 @@
       <c r="G333" t="b">
         <v>0</v>
       </c>
-      <c r="H333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -15150,7 +15071,6 @@
       <c r="G334" t="b">
         <v>0</v>
       </c>
-      <c r="H334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -15184,7 +15104,6 @@
       <c r="G335" t="b">
         <v>0</v>
       </c>
-      <c r="H335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -15218,7 +15137,6 @@
       <c r="G336" t="b">
         <v>0</v>
       </c>
-      <c r="H336" t="inlineStr"/>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -15252,7 +15170,6 @@
       <c r="G337" t="b">
         <v>0</v>
       </c>
-      <c r="H337" t="inlineStr"/>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
@@ -15286,7 +15203,6 @@
       <c r="G338" t="b">
         <v>0</v>
       </c>
-      <c r="H338" t="inlineStr"/>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -15320,7 +15236,6 @@
       <c r="G339" t="b">
         <v>0</v>
       </c>
-      <c r="H339" t="inlineStr"/>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -15354,7 +15269,6 @@
       <c r="G340" t="b">
         <v>0</v>
       </c>
-      <c r="H340" t="inlineStr"/>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -15388,7 +15302,6 @@
       <c r="G341" t="b">
         <v>0</v>
       </c>
-      <c r="H341" t="inlineStr"/>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -15422,7 +15335,6 @@
       <c r="G342" t="b">
         <v>0</v>
       </c>
-      <c r="H342" t="inlineStr"/>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
@@ -15456,7 +15368,6 @@
       <c r="G343" t="b">
         <v>0</v>
       </c>
-      <c r="H343" t="inlineStr"/>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
@@ -15490,7 +15401,6 @@
       <c r="G344" t="b">
         <v>1</v>
       </c>
-      <c r="H344" t="inlineStr"/>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
@@ -15524,7 +15434,6 @@
       <c r="G345" t="b">
         <v>1</v>
       </c>
-      <c r="H345" t="inlineStr"/>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -15558,7 +15467,6 @@
       <c r="G346" t="b">
         <v>1</v>
       </c>
-      <c r="H346" t="inlineStr"/>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
@@ -15592,7 +15500,6 @@
       <c r="G347" t="b">
         <v>1</v>
       </c>
-      <c r="H347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -15626,7 +15533,6 @@
       <c r="G348" t="b">
         <v>1</v>
       </c>
-      <c r="H348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -15660,7 +15566,6 @@
       <c r="G349" t="b">
         <v>1</v>
       </c>
-      <c r="H349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -15694,7 +15599,6 @@
       <c r="G350" t="b">
         <v>1</v>
       </c>
-      <c r="H350" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -15728,7 +15632,6 @@
       <c r="G351" t="b">
         <v>1</v>
       </c>
-      <c r="H351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -15762,7 +15665,6 @@
       <c r="G352" t="b">
         <v>1</v>
       </c>
-      <c r="H352" t="inlineStr"/>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
@@ -15796,7 +15698,6 @@
       <c r="G353" t="b">
         <v>1</v>
       </c>
-      <c r="H353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -15830,7 +15731,6 @@
       <c r="G354" t="b">
         <v>1</v>
       </c>
-      <c r="H354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -15864,7 +15764,6 @@
       <c r="G355" t="b">
         <v>1</v>
       </c>
-      <c r="H355" t="inlineStr"/>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -15898,7 +15797,6 @@
       <c r="G356" t="b">
         <v>1</v>
       </c>
-      <c r="H356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -15932,7 +15830,6 @@
       <c r="G357" t="b">
         <v>1</v>
       </c>
-      <c r="H357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -15966,7 +15863,6 @@
       <c r="G358" t="b">
         <v>1</v>
       </c>
-      <c r="H358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -16000,7 +15896,6 @@
       <c r="G359" t="b">
         <v>1</v>
       </c>
-      <c r="H359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -16034,7 +15929,6 @@
       <c r="G360" t="b">
         <v>1</v>
       </c>
-      <c r="H360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -16068,7 +15962,6 @@
       <c r="G361" t="b">
         <v>1</v>
       </c>
-      <c r="H361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -16102,7 +15995,6 @@
       <c r="G362" t="b">
         <v>1</v>
       </c>
-      <c r="H362" t="inlineStr"/>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
@@ -16136,7 +16028,6 @@
       <c r="G363" t="b">
         <v>1</v>
       </c>
-      <c r="H363" t="inlineStr"/>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
@@ -16170,7 +16061,6 @@
       <c r="G364" t="b">
         <v>1</v>
       </c>
-      <c r="H364" t="inlineStr"/>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
@@ -16204,7 +16094,6 @@
       <c r="G365" t="b">
         <v>1</v>
       </c>
-      <c r="H365" t="inlineStr"/>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
@@ -16238,7 +16127,6 @@
       <c r="G366" t="b">
         <v>1</v>
       </c>
-      <c r="H366" t="inlineStr"/>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
@@ -16272,7 +16160,6 @@
       <c r="G367" t="b">
         <v>1</v>
       </c>
-      <c r="H367" t="inlineStr"/>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
@@ -19438,7 +19325,6 @@
       <c r="G455" t="b">
         <v>0</v>
       </c>
-      <c r="H455" t="inlineStr"/>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
@@ -19472,7 +19358,6 @@
       <c r="G456" t="b">
         <v>0</v>
       </c>
-      <c r="H456" t="inlineStr"/>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
@@ -19506,7 +19391,6 @@
       <c r="G457" t="b">
         <v>0</v>
       </c>
-      <c r="H457" t="inlineStr"/>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
@@ -19540,7 +19424,6 @@
       <c r="G458" t="b">
         <v>0</v>
       </c>
-      <c r="H458" t="inlineStr"/>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
@@ -19574,7 +19457,6 @@
       <c r="G459" t="b">
         <v>0</v>
       </c>
-      <c r="H459" t="inlineStr"/>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
@@ -19608,7 +19490,6 @@
       <c r="G460" t="b">
         <v>0</v>
       </c>
-      <c r="H460" t="inlineStr"/>
     </row>
     <row r="461">
       <c r="A461" t="inlineStr">
@@ -19642,7 +19523,6 @@
       <c r="G461" t="b">
         <v>0</v>
       </c>
-      <c r="H461" t="inlineStr"/>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
@@ -19676,7 +19556,6 @@
       <c r="G462" t="b">
         <v>0</v>
       </c>
-      <c r="H462" t="inlineStr"/>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
@@ -19710,7 +19589,6 @@
       <c r="G463" t="b">
         <v>0</v>
       </c>
-      <c r="H463" t="inlineStr"/>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
@@ -19744,7 +19622,6 @@
       <c r="G464" t="b">
         <v>0</v>
       </c>
-      <c r="H464" t="inlineStr"/>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
@@ -19778,7 +19655,6 @@
       <c r="G465" t="b">
         <v>0</v>
       </c>
-      <c r="H465" t="inlineStr"/>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
@@ -19812,7 +19688,6 @@
       <c r="G466" t="b">
         <v>0</v>
       </c>
-      <c r="H466" t="inlineStr"/>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
@@ -19846,7 +19721,6 @@
       <c r="G467" t="b">
         <v>0</v>
       </c>
-      <c r="H467" t="inlineStr"/>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
@@ -19880,7 +19754,6 @@
       <c r="G468" t="b">
         <v>0</v>
       </c>
-      <c r="H468" t="inlineStr"/>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
@@ -19914,7 +19787,6 @@
       <c r="G469" t="b">
         <v>0</v>
       </c>
-      <c r="H469" t="inlineStr"/>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
@@ -19948,7 +19820,6 @@
       <c r="G470" t="b">
         <v>0</v>
       </c>
-      <c r="H470" t="inlineStr"/>
     </row>
     <row r="471">
       <c r="A471" t="inlineStr">
@@ -19982,7 +19853,6 @@
       <c r="G471" t="b">
         <v>0</v>
       </c>
-      <c r="H471" t="inlineStr"/>
     </row>
     <row r="472">
       <c r="A472" t="inlineStr">
@@ -20016,7 +19886,6 @@
       <c r="G472" t="b">
         <v>0</v>
       </c>
-      <c r="H472" t="inlineStr"/>
     </row>
     <row r="473">
       <c r="A473" t="inlineStr">
@@ -20050,7 +19919,6 @@
       <c r="G473" t="b">
         <v>0</v>
       </c>
-      <c r="H473" t="inlineStr"/>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
@@ -20084,7 +19952,6 @@
       <c r="G474" t="b">
         <v>0</v>
       </c>
-      <c r="H474" t="inlineStr"/>
     </row>
     <row r="475">
       <c r="A475" t="inlineStr">
@@ -20118,7 +19985,6 @@
       <c r="G475" t="b">
         <v>0</v>
       </c>
-      <c r="H475" t="inlineStr"/>
     </row>
     <row r="476">
       <c r="A476" t="inlineStr">
@@ -20152,7 +20018,6 @@
       <c r="G476" t="b">
         <v>0</v>
       </c>
-      <c r="H476" t="inlineStr"/>
     </row>
     <row r="477">
       <c r="A477" t="inlineStr">
@@ -20186,7 +20051,6 @@
       <c r="G477" t="b">
         <v>0</v>
       </c>
-      <c r="H477" t="inlineStr"/>
     </row>
     <row r="478">
       <c r="A478" t="inlineStr">
@@ -20220,7 +20084,6 @@
       <c r="G478" t="b">
         <v>0</v>
       </c>
-      <c r="H478" t="inlineStr"/>
     </row>
     <row r="479">
       <c r="A479" t="inlineStr">
@@ -20254,7 +20117,6 @@
       <c r="G479" t="b">
         <v>0</v>
       </c>
-      <c r="H479" t="inlineStr"/>
     </row>
     <row r="480">
       <c r="A480" t="inlineStr">
@@ -20288,7 +20150,6 @@
       <c r="G480" t="b">
         <v>0</v>
       </c>
-      <c r="H480" t="inlineStr"/>
     </row>
     <row r="481">
       <c r="A481" t="inlineStr">
@@ -20322,7 +20183,6 @@
       <c r="G481" t="b">
         <v>0</v>
       </c>
-      <c r="H481" t="inlineStr"/>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
@@ -20356,7 +20216,6 @@
       <c r="G482" t="b">
         <v>0</v>
       </c>
-      <c r="H482" t="inlineStr"/>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
@@ -20390,7 +20249,6 @@
       <c r="G483" t="b">
         <v>0</v>
       </c>
-      <c r="H483" t="inlineStr"/>
     </row>
     <row r="484">
       <c r="A484" t="inlineStr">
@@ -20424,7 +20282,6 @@
       <c r="G484" t="b">
         <v>0</v>
       </c>
-      <c r="H484" t="inlineStr"/>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
@@ -20458,7 +20315,6 @@
       <c r="G485" t="b">
         <v>0</v>
       </c>
-      <c r="H485" t="inlineStr"/>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
@@ -20492,7 +20348,6 @@
       <c r="G486" t="b">
         <v>0</v>
       </c>
-      <c r="H486" t="inlineStr"/>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
@@ -20526,7 +20381,6 @@
       <c r="G487" t="b">
         <v>0</v>
       </c>
-      <c r="H487" t="inlineStr"/>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
@@ -20560,7 +20414,6 @@
       <c r="G488" t="b">
         <v>0</v>
       </c>
-      <c r="H488" t="inlineStr"/>
     </row>
     <row r="489">
       <c r="A489" t="inlineStr">
@@ -20594,7 +20447,6 @@
       <c r="G489" t="b">
         <v>0</v>
       </c>
-      <c r="H489" t="inlineStr"/>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
@@ -20628,7 +20480,6 @@
       <c r="G490" t="b">
         <v>0</v>
       </c>
-      <c r="H490" t="inlineStr"/>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
@@ -20662,7 +20513,6 @@
       <c r="G491" t="b">
         <v>0</v>
       </c>
-      <c r="H491" t="inlineStr"/>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr">
@@ -20696,7 +20546,6 @@
       <c r="G492" t="b">
         <v>0</v>
       </c>
-      <c r="H492" t="inlineStr"/>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
@@ -20730,7 +20579,6 @@
       <c r="G493" t="b">
         <v>0</v>
       </c>
-      <c r="H493" t="inlineStr"/>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
@@ -20764,7 +20612,6 @@
       <c r="G494" t="b">
         <v>0</v>
       </c>
-      <c r="H494" t="inlineStr"/>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
@@ -20798,7 +20645,6 @@
       <c r="G495" t="b">
         <v>0</v>
       </c>
-      <c r="H495" t="inlineStr"/>
     </row>
     <row r="496">
       <c r="A496" t="inlineStr">
@@ -20832,7 +20678,6 @@
       <c r="G496" t="b">
         <v>0</v>
       </c>
-      <c r="H496" t="inlineStr"/>
     </row>
     <row r="497">
       <c r="A497" t="inlineStr">
@@ -20866,7 +20711,6 @@
       <c r="G497" t="b">
         <v>0</v>
       </c>
-      <c r="H497" t="inlineStr"/>
     </row>
     <row r="498">
       <c r="A498" t="inlineStr">
@@ -20900,7 +20744,6 @@
       <c r="G498" t="b">
         <v>0</v>
       </c>
-      <c r="H498" t="inlineStr"/>
     </row>
     <row r="499">
       <c r="A499" t="inlineStr">
@@ -20934,7 +20777,6 @@
       <c r="G499" t="b">
         <v>0</v>
       </c>
-      <c r="H499" t="inlineStr"/>
     </row>
     <row r="500">
       <c r="A500" t="inlineStr">
@@ -22012,7 +21854,6 @@
       <c r="G529" t="b">
         <v>0</v>
       </c>
-      <c r="H529" t="inlineStr"/>
     </row>
     <row r="530">
       <c r="A530" t="inlineStr">
@@ -22046,7 +21887,6 @@
       <c r="G530" t="b">
         <v>0</v>
       </c>
-      <c r="H530" t="inlineStr"/>
     </row>
     <row r="531">
       <c r="A531" t="inlineStr">
@@ -22080,7 +21920,6 @@
       <c r="G531" t="b">
         <v>0</v>
       </c>
-      <c r="H531" t="inlineStr"/>
     </row>
     <row r="532">
       <c r="A532" t="inlineStr">
@@ -22114,7 +21953,6 @@
       <c r="G532" t="b">
         <v>0</v>
       </c>
-      <c r="H532" t="inlineStr"/>
     </row>
     <row r="533">
       <c r="A533" t="inlineStr">
@@ -22148,7 +21986,6 @@
       <c r="G533" t="b">
         <v>0</v>
       </c>
-      <c r="H533" t="inlineStr"/>
     </row>
     <row r="534">
       <c r="A534" t="inlineStr">
@@ -22182,7 +22019,6 @@
       <c r="G534" t="b">
         <v>0</v>
       </c>
-      <c r="H534" t="inlineStr"/>
     </row>
     <row r="535">
       <c r="A535" t="inlineStr">
@@ -22216,7 +22052,6 @@
       <c r="G535" t="b">
         <v>0</v>
       </c>
-      <c r="H535" t="inlineStr"/>
     </row>
     <row r="536">
       <c r="A536" t="inlineStr">
@@ -22250,7 +22085,6 @@
       <c r="G536" t="b">
         <v>0</v>
       </c>
-      <c r="H536" t="inlineStr"/>
     </row>
     <row r="537">
       <c r="A537" t="inlineStr">
@@ -22284,7 +22118,6 @@
       <c r="G537" t="b">
         <v>0</v>
       </c>
-      <c r="H537" t="inlineStr"/>
     </row>
     <row r="538">
       <c r="A538" t="inlineStr">
@@ -22318,7 +22151,6 @@
       <c r="G538" t="b">
         <v>0</v>
       </c>
-      <c r="H538" t="inlineStr"/>
     </row>
     <row r="539">
       <c r="A539" t="inlineStr">
@@ -22352,7 +22184,6 @@
       <c r="G539" t="b">
         <v>0</v>
       </c>
-      <c r="H539" t="inlineStr"/>
     </row>
     <row r="540">
       <c r="A540" t="inlineStr">
@@ -22386,7 +22217,6 @@
       <c r="G540" t="b">
         <v>0</v>
       </c>
-      <c r="H540" t="inlineStr"/>
     </row>
     <row r="541">
       <c r="A541" t="inlineStr">
@@ -22420,7 +22250,6 @@
       <c r="G541" t="b">
         <v>0</v>
       </c>
-      <c r="H541" t="inlineStr"/>
     </row>
     <row r="542">
       <c r="A542" t="inlineStr">
@@ -22454,7 +22283,6 @@
       <c r="G542" t="b">
         <v>0</v>
       </c>
-      <c r="H542" t="inlineStr"/>
     </row>
     <row r="543">
       <c r="A543" t="inlineStr">
@@ -22488,7 +22316,6 @@
       <c r="G543" t="b">
         <v>0</v>
       </c>
-      <c r="H543" t="inlineStr"/>
     </row>
     <row r="544">
       <c r="A544" t="inlineStr">
@@ -22522,7 +22349,6 @@
       <c r="G544" t="b">
         <v>0</v>
       </c>
-      <c r="H544" t="inlineStr"/>
     </row>
     <row r="545">
       <c r="A545" t="inlineStr">
@@ -22556,7 +22382,6 @@
       <c r="G545" t="b">
         <v>0</v>
       </c>
-      <c r="H545" t="inlineStr"/>
     </row>
     <row r="546">
       <c r="A546" t="inlineStr">
@@ -22590,7 +22415,6 @@
       <c r="G546" t="b">
         <v>0</v>
       </c>
-      <c r="H546" t="inlineStr"/>
     </row>
     <row r="547">
       <c r="A547" t="inlineStr">
@@ -22624,7 +22448,6 @@
       <c r="G547" t="b">
         <v>0</v>
       </c>
-      <c r="H547" t="inlineStr"/>
     </row>
     <row r="548">
       <c r="A548" t="inlineStr">
@@ -22658,7 +22481,6 @@
       <c r="G548" t="b">
         <v>0</v>
       </c>
-      <c r="H548" t="inlineStr"/>
     </row>
     <row r="549">
       <c r="A549" t="inlineStr">
@@ -22692,7 +22514,6 @@
       <c r="G549" t="b">
         <v>0</v>
       </c>
-      <c r="H549" t="inlineStr"/>
     </row>
     <row r="550">
       <c r="A550" t="inlineStr">
@@ -32987,1556 +32808,149 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J41"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>var</t>
+          <t>label</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>company</t>
+          <t>beta</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>fy</t>
+          <t>p</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>q</t>
+          <t>n</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>computed</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>found</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>student_checked_value</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>matches_source_YN</t>
+          <t>firms</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>AAVAS Financiers Ltd.</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>FY23</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
+          <t>All firms (main)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>-3.293171437825413</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.27996399819991</v>
+      </c>
+      <c r="D2" t="n">
+        <v>235</v>
       </c>
       <c r="E2" t="n">
-        <v>7.29</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>24-2 p.21</t>
-        </is>
-      </c>
-      <c r="G2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
+        <v>15</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Arman Financial Services Ltd.</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>FY22</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
+          <t>Excluding IIFL Finance (gold-loan embargo Mar-Sep 2024)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>-3.405794303008516</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.2846642332116606</v>
+      </c>
+      <c r="D3" t="n">
+        <v>230</v>
       </c>
       <c r="E3" t="n">
-        <v>12.05</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>22-3 P&amp;L + borrowing-mix chart</t>
-        </is>
-      </c>
-      <c r="G3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
+        <v>14</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Arman Financial Services Ltd.</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
+          <t>Excluding NBFC-MFIs (CreditAccess, Arman: bank loans largely priority-sector, exempt)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>-3.35146571290758</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.3908195409770489</v>
+      </c>
+      <c r="D4" t="n">
+        <v>198</v>
       </c>
       <c r="E4" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>25-2 p.24</t>
-        </is>
-      </c>
-      <c r="G4" t="b">
-        <v>0</v>
-      </c>
-      <c r="H4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
+        <v>13</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Bajaj Finance Ltd.</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>FY22</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
+          <t>Excluding IIFL and NBFC-MFIs</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>-3.504598533192995</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.3929696484824241</v>
+      </c>
+      <c r="D5" t="n">
+        <v>193</v>
       </c>
       <c r="E5" t="n">
-        <v>29</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>22-3 lead indicators</t>
-        </is>
-      </c>
-      <c r="G5" t="b">
-        <v>0</v>
-      </c>
-      <c r="H5" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr"/>
+        <v>12</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Bajaj Finance Ltd.</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>FY23</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
+          <t>Excluding IIFL, NBFC-MFIs and Muthoot</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>-4.037947254891492</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.4036201810090504</v>
+      </c>
+      <c r="D6" t="n">
+        <v>173</v>
       </c>
       <c r="E6" t="n">
-        <v>33</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>23-4 lead indicators</t>
-        </is>
-      </c>
-      <c r="G6" t="b">
-        <v>0</v>
-      </c>
-      <c r="H6" t="b">
-        <v>1</v>
-      </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
+        <v>11</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Bajaj Finance Ltd.</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
+          <t>Excluding SBI Cards</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>-5.153058134140627</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.05610280514025701</v>
+      </c>
+      <c r="D7" t="n">
+        <v>217</v>
       </c>
       <c r="E7" t="n">
-        <v>7.96</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>25-3 lead indicators (BFL standalone)</t>
-        </is>
-      </c>
-      <c r="G7" t="b">
-        <v>0</v>
-      </c>
-      <c r="H7" t="b">
-        <v>1</v>
-      </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Bajaj Finance Ltd.</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>29</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>25-3 lead indicators</t>
-        </is>
-      </c>
-      <c r="G8" t="b">
-        <v>0</v>
-      </c>
-      <c r="H8" t="b">
-        <v>1</v>
-      </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Bajaj Finance Ltd.</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>FY26</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>7.41</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>26-4 lead indicators (BFL standalone)</t>
-        </is>
-      </c>
-      <c r="G9" t="b">
-        <v>0</v>
-      </c>
-      <c r="H9" t="b">
-        <v>1</v>
-      </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Can Fin Homes Ltd.</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>FY23</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>23-1</t>
-        </is>
-      </c>
-      <c r="G10" t="b">
-        <v>0</v>
-      </c>
-      <c r="H10" t="b">
-        <v>1</v>
-      </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Can Fin Homes Ltd.</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>FY23</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>54</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>24-2 funding basket pies</t>
-        </is>
-      </c>
-      <c r="G11" t="b">
-        <v>0</v>
-      </c>
-      <c r="H11" t="b">
-        <v>1</v>
-      </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Can Fin Homes Ltd.</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>7.56</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>25-2</t>
-        </is>
-      </c>
-      <c r="G12" t="b">
-        <v>0</v>
-      </c>
-      <c r="H12" t="b">
-        <v>1</v>
-      </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Cholamandalam Investment &amp; Finance Company Ltd.</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>FY23</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>66</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>23-4 p.67</t>
-        </is>
-      </c>
-      <c r="G13" t="b">
-        <v>0</v>
-      </c>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Cholamandalam Investment &amp; Finance Company Ltd.</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>FY23</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>64</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>23-4 p.67</t>
-        </is>
-      </c>
-      <c r="G14" t="b">
-        <v>0</v>
-      </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Cholamandalam Investment &amp; Finance Company Ltd.</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>7.1</v>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>26-4 total-company P&amp;L table</t>
-        </is>
-      </c>
-      <c r="G15" t="b">
-        <v>1</v>
-      </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Cholamandalam Investment &amp; Finance Company Ltd.</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>58</v>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>25-4 p.72 (banks+IFI)</t>
-        </is>
-      </c>
-      <c r="G16" t="b">
-        <v>0</v>
-      </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Cholamandalam Investment &amp; Finance Company Ltd.</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>FY26</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>59</v>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>26-4 p.76 (banks+IFI)</t>
-        </is>
-      </c>
-      <c r="G17" t="b">
-        <v>0</v>
-      </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>CreditAccess Grameen Ltd.</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>FY21</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>21-2 key ratios (or 5-quarter key metrics in FY23-25 decks)</t>
-        </is>
-      </c>
-      <c r="G18" t="b">
-        <v>0</v>
-      </c>
-      <c r="H18" t="b">
-        <v>1</v>
-      </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>CreditAccess Grameen Ltd.</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>FY21</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>52.1</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>21-4 liability mix pie</t>
-        </is>
-      </c>
-      <c r="G19" t="b">
-        <v>0</v>
-      </c>
-      <c r="H19" t="b">
-        <v>1</v>
-      </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>CreditAccess Grameen Ltd.</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>FY22</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>49.5</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>22-2 liability mix pie</t>
-        </is>
-      </c>
-      <c r="G20" t="b">
-        <v>0</v>
-      </c>
-      <c r="H20" t="b">
-        <v>1</v>
-      </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>CreditAccess Grameen Ltd.</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>9.800000000000001</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>24-2 key ratios (or 5-quarter key metrics in FY23-25 decks)</t>
-        </is>
-      </c>
-      <c r="G21" t="b">
-        <v>0</v>
-      </c>
-      <c r="H21" t="b">
-        <v>1</v>
-      </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Home First Finance Company India Ltd.</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>FY21</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>22-1 p.24 chart</t>
-        </is>
-      </c>
-      <c r="G22" t="b">
-        <v>0</v>
-      </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Home First Finance Company India Ltd.</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>FY24</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>8</v>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>24-2 p.31 chart</t>
-        </is>
-      </c>
-      <c r="G23" t="b">
-        <v>0</v>
-      </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>LIC Housing Finance Ltd.</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>FY22</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>30</v>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>22-4 liability profile pie</t>
-        </is>
-      </c>
-      <c r="G24" t="b">
-        <v>0</v>
-      </c>
-      <c r="H24" t="b">
-        <v>1</v>
-      </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>LIC Housing Finance Ltd.</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>7.76</v>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>25-1 key financials</t>
-        </is>
-      </c>
-      <c r="G25" t="b">
-        <v>0</v>
-      </c>
-      <c r="H25" t="b">
-        <v>1</v>
-      </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Mahindra &amp; Mahindra Financial Services Ltd.</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>FY22</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="E26" t="n">
-        <v>45.3</v>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>22-2 funding mix by investor category</t>
-        </is>
-      </c>
-      <c r="G26" t="b">
-        <v>0</v>
-      </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Mahindra &amp; Mahindra Financial Services Ltd.</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>FY22</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>6.61</v>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>22-4 P&amp;L + funding mix</t>
-        </is>
-      </c>
-      <c r="G27" t="b">
-        <v>1</v>
-      </c>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Mahindra &amp; Mahindra Financial Services Ltd.</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>60</v>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>25-3 funding mix by investor category</t>
-        </is>
-      </c>
-      <c r="G28" t="b">
-        <v>0</v>
-      </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Muthoot Finance Ltd.</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>FY22</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="E29" t="n">
-        <v>8.15</v>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>22-4 highlights</t>
-        </is>
-      </c>
-      <c r="G29" t="b">
-        <v>0</v>
-      </c>
-      <c r="H29" t="b">
-        <v>1</v>
-      </c>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Muthoot Finance Ltd.</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>FY23</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
-      </c>
-      <c r="E30" t="n">
-        <v>55.9</v>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>23-2 stable sources of funding</t>
-        </is>
-      </c>
-      <c r="G30" t="b">
-        <v>0</v>
-      </c>
-      <c r="H30" t="b">
-        <v>0</v>
-      </c>
-      <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Muthoot Finance Ltd.</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="E31" t="n">
-        <v>8.92</v>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>25-3 highlights</t>
-        </is>
-      </c>
-      <c r="G31" t="b">
-        <v>0</v>
-      </c>
-      <c r="H31" t="b">
-        <v>1</v>
-      </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>PNB Housing Finance Ltd.</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="E32" t="n">
-        <v>7.84</v>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>26-1 (prior qtr)</t>
-        </is>
-      </c>
-      <c r="G32" t="b">
-        <v>0</v>
-      </c>
-      <c r="H32" t="b">
-        <v>1</v>
-      </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Poonawalla Fincorp Ltd.</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="E33" t="n">
-        <v>8.06</v>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>26-2 p.24 chart</t>
-        </is>
-      </c>
-      <c r="G33" t="b">
-        <v>0</v>
-      </c>
-      <c r="H33" t="b">
-        <v>1</v>
-      </c>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Repco Home Finance Ltd.</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>FY22</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>7</v>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>22-1 quarterly results table</t>
-        </is>
-      </c>
-      <c r="G34" t="b">
-        <v>0</v>
-      </c>
-      <c r="H34" t="b">
-        <v>1</v>
-      </c>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Repco Home Finance Ltd.</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>FY23</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
-      <c r="E35" t="n">
-        <v>71</v>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>23-1 borrowing profile</t>
-        </is>
-      </c>
-      <c r="G35" t="b">
-        <v>0</v>
-      </c>
-      <c r="H35" t="b">
-        <v>1</v>
-      </c>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Repco Home Finance Ltd.</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>FY23</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>72.09999999999999</v>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>23-3 borrowing profile</t>
-        </is>
-      </c>
-      <c r="G36" t="b">
-        <v>0</v>
-      </c>
-      <c r="H36" t="b">
-        <v>0</v>
-      </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>Repco Home Finance Ltd.</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>79.8</v>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>25-1 borrowing profile</t>
-        </is>
-      </c>
-      <c r="G37" t="b">
-        <v>0</v>
-      </c>
-      <c r="H37" t="b">
-        <v>1</v>
-      </c>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>SBI Cards and Payment Services Ltd.</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>FY22</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="E38" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>22-4 p.14</t>
-        </is>
-      </c>
-      <c r="G38" t="b">
-        <v>0</v>
-      </c>
-      <c r="H38" t="b">
-        <v>1</v>
-      </c>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Bank share</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>SBI Cards and Payment Services Ltd.</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>FY26</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>86</v>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>26-4 p.17</t>
-        </is>
-      </c>
-      <c r="G39" t="b">
-        <v>0</v>
-      </c>
-      <c r="H39" t="b">
-        <v>1</v>
-      </c>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>SBI Cards and Payment Services Ltd.</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>FY26</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>26-4 key metrics</t>
-        </is>
-      </c>
-      <c r="G40" t="b">
-        <v>0</v>
-      </c>
-      <c r="H40" t="b">
-        <v>1</v>
-      </c>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>COF</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>Shriram Finance Ltd.</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="E41" t="n">
-        <v>8.869999999999999</v>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>23-4/24-4/25-4/26-4 P&amp;L + borrowing profile</t>
-        </is>
-      </c>
-      <c r="G41" t="b">
-        <v>1</v>
-      </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
+        <v>14</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -34549,13 +32963,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>label</t>
+          <t>block</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
@@ -34565,132 +32979,287 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>lo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>p</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>firms</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>All firms (main)</t>
-        </is>
+      <c r="A2" t="n">
+        <v>-11</v>
       </c>
       <c r="B2" t="n">
-        <v>-3.293171437825413</v>
+        <v>-2.968269204295443</v>
       </c>
       <c r="C2" t="n">
-        <v>0.27996399819991</v>
+        <v>-4.191453406561572</v>
       </c>
       <c r="D2" t="n">
-        <v>235</v>
+        <v>-1.745085002029315</v>
       </c>
       <c r="E2" t="n">
-        <v>15</v>
+        <v>2.638321344697661e-05</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Excluding IIFL Finance (gold-loan embargo Mar-Sep 2024)</t>
-        </is>
+      <c r="A3" t="n">
+        <v>-10</v>
       </c>
       <c r="B3" t="n">
-        <v>-3.405794303008516</v>
+        <v>0.9269339761816067</v>
       </c>
       <c r="C3" t="n">
-        <v>0.2846642332116606</v>
+        <v>-0.7331514585098673</v>
       </c>
       <c r="D3" t="n">
-        <v>230</v>
+        <v>2.587019410873081</v>
       </c>
       <c r="E3" t="n">
-        <v>14</v>
+        <v>0.2631696051574309</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Excluding NBFC-MFIs (CreditAccess, Arman: bank loans largely priority-sector, exempt)</t>
-        </is>
+      <c r="A4" t="n">
+        <v>-9</v>
       </c>
       <c r="B4" t="n">
-        <v>-3.35146571290758</v>
+        <v>-0.04323083753365093</v>
       </c>
       <c r="C4" t="n">
-        <v>0.3908195409770489</v>
+        <v>-1.375570245370317</v>
       </c>
       <c r="D4" t="n">
-        <v>198</v>
+        <v>1.289108570303015</v>
       </c>
       <c r="E4" t="n">
-        <v>13</v>
+        <v>0.9476054954401949</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Excluding IIFL and NBFC-MFIs</t>
-        </is>
+      <c r="A5" t="n">
+        <v>-8</v>
       </c>
       <c r="B5" t="n">
-        <v>-3.504598533192995</v>
+        <v>-0.653738585266802</v>
       </c>
       <c r="C5" t="n">
-        <v>0.3929696484824241</v>
+        <v>-1.699294504611323</v>
       </c>
       <c r="D5" t="n">
-        <v>193</v>
+        <v>0.3918173340777186</v>
       </c>
       <c r="E5" t="n">
-        <v>12</v>
+        <v>0.211418909326138</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Excluding IIFL, NBFC-MFIs and Muthoot</t>
-        </is>
+      <c r="A6" t="n">
+        <v>-7</v>
       </c>
       <c r="B6" t="n">
-        <v>-4.037947254891492</v>
+        <v>0.6315065301507361</v>
       </c>
       <c r="C6" t="n">
-        <v>0.4036201810090504</v>
+        <v>-0.5363737068841439</v>
       </c>
       <c r="D6" t="n">
-        <v>173</v>
+        <v>1.799386767185616</v>
       </c>
       <c r="E6" t="n">
-        <v>11</v>
+        <v>0.2782351952262957</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Excluding SBI Cards</t>
-        </is>
+      <c r="A7" t="n">
+        <v>-6</v>
       </c>
       <c r="B7" t="n">
-        <v>-5.153058134140627</v>
+        <v>-0.320417691501667</v>
       </c>
       <c r="C7" t="n">
-        <v>0.05610280514025701</v>
+        <v>-1.668849617801717</v>
       </c>
       <c r="D7" t="n">
-        <v>217</v>
+        <v>1.028014234798383</v>
       </c>
       <c r="E7" t="n">
-        <v>14</v>
+        <v>0.6309960442631312</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>-5</v>
+      </c>
+      <c r="B8" t="n">
+        <v>-0.544584747970086</v>
+      </c>
+      <c r="C8" t="n">
+        <v>-1.929153092257645</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.8399835963174731</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.4281340984281889</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>-4</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.1350978842587351</v>
+      </c>
+      <c r="C9" t="n">
+        <v>-0.9085066599861105</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1.178702428503581</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.7932960831913566</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>-3</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.3728320703685263</v>
+      </c>
+      <c r="C10" t="n">
+        <v>-1.137521929235157</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1.88318606997221</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.6178480205812129</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>-2</v>
+      </c>
+      <c r="B11" t="n">
+        <v>-0.459897136206747</v>
+      </c>
+      <c r="C11" t="n">
+        <v>-1.595651646895925</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.6758573744824314</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.4147834194703851</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>-1</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>0</v>
+      </c>
+      <c r="B13" t="n">
+        <v>-0.6285229220040277</v>
+      </c>
+      <c r="C13" t="n">
+        <v>-1.559557016037318</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.302511172029262</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.1781823130298957</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B14" t="n">
+        <v>-0.9951225678348344</v>
+      </c>
+      <c r="C14" t="n">
+        <v>-2.181626370752665</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.1913812350829963</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.09705752905595283</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" t="n">
+        <v>-1.126641343256956</v>
+      </c>
+      <c r="C15" t="n">
+        <v>-2.260405958977376</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.007123272463465113</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.05136604750362124</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" t="n">
+        <v>-0.6949260978641802</v>
+      </c>
+      <c r="C16" t="n">
+        <v>-2.136599909892209</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.7467477141638486</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.3327769450055734</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" t="n">
+        <v>-1.367407800039115</v>
+      </c>
+      <c r="C17" t="n">
+        <v>-2.393708701584281</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-0.3411068984939487</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.01072586903444517</v>
       </c>
     </row>
   </sheetData>
@@ -34739,16 +33308,16 @@
         <v>-11</v>
       </c>
       <c r="B2" t="n">
-        <v>-2.968269204295443</v>
+        <v>-3.66272526016044</v>
       </c>
       <c r="C2" t="n">
-        <v>-4.191453406561572</v>
+        <v>-4.65598592776109</v>
       </c>
       <c r="D2" t="n">
-        <v>-1.745085002029315</v>
+        <v>-2.669464592559789</v>
       </c>
       <c r="E2" t="n">
-        <v>2.638321344697661e-05</v>
+        <v>2.587297829982871e-08</v>
       </c>
     </row>
     <row r="3">
@@ -34756,16 +33325,16 @@
         <v>-10</v>
       </c>
       <c r="B3" t="n">
-        <v>0.9269339761816067</v>
+        <v>-2.237863292832703</v>
       </c>
       <c r="C3" t="n">
-        <v>-0.7331514585098673</v>
+        <v>-3.050644490695948</v>
       </c>
       <c r="D3" t="n">
-        <v>2.587019410873081</v>
+        <v>-1.425082094969458</v>
       </c>
       <c r="E3" t="n">
-        <v>0.2631696051574309</v>
+        <v>4.399831142713284e-06</v>
       </c>
     </row>
     <row r="4">
@@ -34773,16 +33342,16 @@
         <v>-9</v>
       </c>
       <c r="B4" t="n">
-        <v>-0.04323083753365093</v>
+        <v>0.2397201116360497</v>
       </c>
       <c r="C4" t="n">
-        <v>-1.375570245370317</v>
+        <v>-0.8828623313008941</v>
       </c>
       <c r="D4" t="n">
-        <v>1.289108570303015</v>
+        <v>1.362302554572993</v>
       </c>
       <c r="E4" t="n">
-        <v>0.9476054954401949</v>
+        <v>0.6655307788122309</v>
       </c>
     </row>
     <row r="5">
@@ -34790,16 +33359,16 @@
         <v>-8</v>
       </c>
       <c r="B5" t="n">
-        <v>-0.653738585266802</v>
+        <v>0.2775541808697207</v>
       </c>
       <c r="C5" t="n">
-        <v>-1.699294504611323</v>
+        <v>-1.55305419067259</v>
       </c>
       <c r="D5" t="n">
-        <v>0.3918173340777186</v>
+        <v>2.108162552412031</v>
       </c>
       <c r="E5" t="n">
-        <v>0.211418909326138</v>
+        <v>0.7587064587702271</v>
       </c>
     </row>
     <row r="6">
@@ -34807,16 +33376,16 @@
         <v>-7</v>
       </c>
       <c r="B6" t="n">
-        <v>0.6315065301507361</v>
+        <v>-1.005005485132612</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.5363737068841439</v>
+        <v>-1.602483525720079</v>
       </c>
       <c r="D6" t="n">
-        <v>1.799386767185616</v>
+        <v>-0.4075274445451457</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2782351952262957</v>
+        <v>0.001783028954882734</v>
       </c>
     </row>
     <row r="7">
@@ -34824,16 +33393,16 @@
         <v>-6</v>
       </c>
       <c r="B7" t="n">
-        <v>-0.320417691501667</v>
+        <v>-0.04509964443588674</v>
       </c>
       <c r="C7" t="n">
-        <v>-1.668849617801717</v>
+        <v>-1.580347135631976</v>
       </c>
       <c r="D7" t="n">
-        <v>1.028014234798383</v>
+        <v>1.490147846760202</v>
       </c>
       <c r="E7" t="n">
-        <v>0.6309960442631312</v>
+        <v>0.9525032961355655</v>
       </c>
     </row>
     <row r="8">
@@ -34841,16 +33410,16 @@
         <v>-5</v>
       </c>
       <c r="B8" t="n">
-        <v>-0.544584747970086</v>
+        <v>1.322616320349882</v>
       </c>
       <c r="C8" t="n">
-        <v>-1.929153092257645</v>
+        <v>0.04131255793896305</v>
       </c>
       <c r="D8" t="n">
-        <v>0.8399835963174731</v>
+        <v>2.603920082760802</v>
       </c>
       <c r="E8" t="n">
-        <v>0.4281340984281889</v>
+        <v>0.04349573924419699</v>
       </c>
     </row>
     <row r="9">
@@ -34858,16 +33427,16 @@
         <v>-4</v>
       </c>
       <c r="B9" t="n">
-        <v>0.1350978842587351</v>
+        <v>0.4907774519791634</v>
       </c>
       <c r="C9" t="n">
-        <v>-0.9085066599861105</v>
+        <v>-1.822614086967215</v>
       </c>
       <c r="D9" t="n">
-        <v>1.178702428503581</v>
+        <v>2.804168990925542</v>
       </c>
       <c r="E9" t="n">
-        <v>0.7932960831913566</v>
+        <v>0.6675807505699017</v>
       </c>
     </row>
     <row r="10">
@@ -34875,16 +33444,16 @@
         <v>-3</v>
       </c>
       <c r="B10" t="n">
-        <v>0.3728320703685263</v>
+        <v>-1.941513254861899</v>
       </c>
       <c r="C10" t="n">
-        <v>-1.137521929235157</v>
+        <v>-2.701024171489715</v>
       </c>
       <c r="D10" t="n">
-        <v>1.88318606997221</v>
+        <v>-1.182002338234083</v>
       </c>
       <c r="E10" t="n">
-        <v>0.6178480205812129</v>
+        <v>1.345381498806699e-05</v>
       </c>
     </row>
     <row r="11">
@@ -34892,16 +33461,16 @@
         <v>-2</v>
       </c>
       <c r="B11" t="n">
-        <v>-0.459897136206747</v>
+        <v>0.6339380492143496</v>
       </c>
       <c r="C11" t="n">
-        <v>-1.595651646895925</v>
+        <v>-0.6832698049200654</v>
       </c>
       <c r="D11" t="n">
-        <v>0.6758573744824314</v>
+        <v>1.951145903348765</v>
       </c>
       <c r="E11" t="n">
-        <v>0.4147834194703851</v>
+        <v>0.3331016054140258</v>
       </c>
     </row>
     <row r="12">
@@ -34917,318 +33486,6 @@
       <c r="D12" t="n">
         <v>0</v>
       </c>
-      <c r="E12" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="n">
-        <v>0</v>
-      </c>
-      <c r="B13" t="n">
-        <v>-0.6285229220040277</v>
-      </c>
-      <c r="C13" t="n">
-        <v>-1.559557016037318</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0.302511172029262</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0.1781823130298957</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B14" t="n">
-        <v>-0.9951225678348344</v>
-      </c>
-      <c r="C14" t="n">
-        <v>-2.181626370752665</v>
-      </c>
-      <c r="D14" t="n">
-        <v>0.1913812350829963</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0.09705752905595283</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="n">
-        <v>2</v>
-      </c>
-      <c r="B15" t="n">
-        <v>-1.126641343256956</v>
-      </c>
-      <c r="C15" t="n">
-        <v>-2.260405958977376</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0.007123272463465113</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0.05136604750362124</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>3</v>
-      </c>
-      <c r="B16" t="n">
-        <v>-0.6949260978641802</v>
-      </c>
-      <c r="C16" t="n">
-        <v>-2.136599909892209</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0.7467477141638486</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0.3327769450055734</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>4</v>
-      </c>
-      <c r="B17" t="n">
-        <v>-1.367407800039115</v>
-      </c>
-      <c r="C17" t="n">
-        <v>-2.393708701584281</v>
-      </c>
-      <c r="D17" t="n">
-        <v>-0.3411068984939487</v>
-      </c>
-      <c r="E17" t="n">
-        <v>0.01072586903444517</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>block</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>beta</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>lo</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>hi</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>p</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>-11</v>
-      </c>
-      <c r="B2" t="n">
-        <v>-3.66272526016044</v>
-      </c>
-      <c r="C2" t="n">
-        <v>-4.65598592776109</v>
-      </c>
-      <c r="D2" t="n">
-        <v>-2.669464592559789</v>
-      </c>
-      <c r="E2" t="n">
-        <v>2.587297829982871e-08</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>-10</v>
-      </c>
-      <c r="B3" t="n">
-        <v>-2.237863292832703</v>
-      </c>
-      <c r="C3" t="n">
-        <v>-3.050644490695948</v>
-      </c>
-      <c r="D3" t="n">
-        <v>-1.425082094969458</v>
-      </c>
-      <c r="E3" t="n">
-        <v>4.399831142713284e-06</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>-9</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.2397201116360497</v>
-      </c>
-      <c r="C4" t="n">
-        <v>-0.8828623313008941</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1.362302554572993</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.6655307788122309</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>-8</v>
-      </c>
-      <c r="B5" t="n">
-        <v>0.2775541808697207</v>
-      </c>
-      <c r="C5" t="n">
-        <v>-1.55305419067259</v>
-      </c>
-      <c r="D5" t="n">
-        <v>2.108162552412031</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0.7587064587702271</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>-7</v>
-      </c>
-      <c r="B6" t="n">
-        <v>-1.005005485132612</v>
-      </c>
-      <c r="C6" t="n">
-        <v>-1.602483525720079</v>
-      </c>
-      <c r="D6" t="n">
-        <v>-0.4075274445451457</v>
-      </c>
-      <c r="E6" t="n">
-        <v>0.001783028954882734</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>-6</v>
-      </c>
-      <c r="B7" t="n">
-        <v>-0.04509964443588674</v>
-      </c>
-      <c r="C7" t="n">
-        <v>-1.580347135631976</v>
-      </c>
-      <c r="D7" t="n">
-        <v>1.490147846760202</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.9525032961355655</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>-5</v>
-      </c>
-      <c r="B8" t="n">
-        <v>1.322616320349882</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.04131255793896305</v>
-      </c>
-      <c r="D8" t="n">
-        <v>2.603920082760802</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0.04349573924419699</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>-4</v>
-      </c>
-      <c r="B9" t="n">
-        <v>0.4907774519791634</v>
-      </c>
-      <c r="C9" t="n">
-        <v>-1.822614086967215</v>
-      </c>
-      <c r="D9" t="n">
-        <v>2.804168990925542</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0.6675807505699017</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="n">
-        <v>-3</v>
-      </c>
-      <c r="B10" t="n">
-        <v>-1.941513254861899</v>
-      </c>
-      <c r="C10" t="n">
-        <v>-2.701024171489715</v>
-      </c>
-      <c r="D10" t="n">
-        <v>-1.182002338234083</v>
-      </c>
-      <c r="E10" t="n">
-        <v>1.345381498806699e-05</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>-2</v>
-      </c>
-      <c r="B11" t="n">
-        <v>0.6339380492143496</v>
-      </c>
-      <c r="C11" t="n">
-        <v>-0.6832698049200654</v>
-      </c>
-      <c r="D11" t="n">
-        <v>1.951145903348765</v>
-      </c>
-      <c r="E11" t="n">
-        <v>0.3331016054140258</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="n">
-        <v>-1</v>
-      </c>
-      <c r="B12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C12" t="n">
-        <v>0</v>
-      </c>
-      <c r="D12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">

</xml_diff>